<commit_message>
Fix inflated per-person total, verify extras/food links, rebuild pages
Section A-C personal-item total was $929.28/person because build_buy_list.py
summed qty*unit_price (whole-group cost, since qty=headcount) into the
per-person personal total instead of unit_price alone. Fixed to accumulate
unit_price; personal total is now $154.88/person.

Replaced Amazon search/category links with verified exact product pages
(BIC lighters, tortillas, tuna pouches, PB packets, trail mix, dish tub,
table cover, panning tweezers/magnet/spray-bottle) via WebFetch/browser
verification, using Walmart where Amazon listings were placeholder/dead
ASINs. Split the combined tuna+PB row into two accurately priced rows.

Rebuilt all generated pages (Gear_Picker.xlsx, BUY_LIST.md, index.html,
gear-checkin.html, RUNDOWN.html/md) from the corrected data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gear_Picker.xlsx
+++ b/Gear_Picker.xlsx
@@ -1090,7 +1090,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Vogel SP Oct 15-21 lows, 2020-2025, averaged 39-48F; the coldest single night was 29F (Oct 2022). NOAA's Oct-Dec 2026 outlook favors a warmer, wetter season (strong El Nino). A 30F-rated bag/quilt plus a puffy and base layer covers this comfortably for most people, and rain protection matters more than an extra 10F of bag rating this year. The 30F group is the RECOMMENDED DEFAULT on the Picker; the existing 20F group is kept as an 'alt' row (backup / more cold margin) rather than deleted.</t>
+          <t>Vogel SP Oct 15-21 lows, 2020-2025, averaged 39-48F; the coldest single night was 29F (Oct 2022). NOAA's Oct-Dec 2026 outlook favors a warmer, wetter season (strong El Nino). A 30F-rated bag/quilt plus a puffy and base layer covers this comfortably for most people, and rain protection matters more than an extra 10F of bag rating this year. The 30F group is the RECOMMENDED DEFAULT on the Picker, specifically the Budget synthetic bag (zippered, no draft-sealing technique needed) -- the Value/Premium quilts in that group are flagged BEGINNER CAUTION and are upgrade options, not the default, since a quilt with an unsealed pad gap can be a cold, unpleasant surprise on a first cold-weather trip. the existing 20F group is kept as an 'alt' row (backup / more cold margin) rather than deleted.</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Tent/shelter (his share, split w/ tentmate)</t>
+          <t>Tent/shelter (shared, split w/ tentmate)</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Sleeping bag/quilt (30F) -- RECOMMENDED default</t>
+          <t>Sleeping bag/quilt (30F) -- RECOMMENDED default, beginner-safe</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Budget</t>
         </is>
       </c>
       <c r="F11" s="10">
@@ -2805,7 +2805,7 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Stove (his share of group stove)</t>
+          <t>Stove (group/shared item)</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>Cook pot (his share)</t>
+          <t>Cook pot (group/shared item)</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Fuel canister (his share)</t>
+          <t>Fuel canister (group/shared item)</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t>Water filter (his share)</t>
+          <t>Water filter (group/shared item)</t>
         </is>
       </c>
       <c r="C25" s="10" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>Bear-proof food storage (his share)</t>
+          <t>Bear-proof food storage (group/shared item)</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>First aid kit (his share, overnight-size)</t>
+          <t>First aid kit (group/shared item, overnight-size)</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>Satellite messenger (his share)</t>
+          <t>Satellite messenger (group/shared item)</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -5815,14 +5815,14 @@
       </c>
       <c r="C3" s="32" t="inlineStr">
         <is>
-          <t>Rook 50 (men's) / Renn 50 (women's)</t>
+          <t>Rook 65 (men's) / Renn 65 (women's)</t>
         </is>
       </c>
       <c r="D3" s="33" t="n">
         <v>66</v>
       </c>
       <c r="E3" s="34" t="n">
-        <v>155</v>
+        <v>205</v>
       </c>
       <c r="F3" s="11" t="inlineStr">
         <is>
@@ -5951,7 +5951,7 @@
         <v>91</v>
       </c>
       <c r="E4" s="34" t="n">
-        <v>159</v>
+        <v>259</v>
       </c>
       <c r="F4" s="11" t="inlineStr">
         <is>
@@ -6029,7 +6029,7 @@
         <v>18.5</v>
       </c>
       <c r="W4" s="34" t="n">
-        <v>699</v>
+        <v>749</v>
       </c>
       <c r="X4" s="11" t="inlineStr">
         <is>
@@ -6073,14 +6073,14 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>Trestles 15 (or Kelty Cosmic 20 Synthetic)</t>
+          <t>Trestles Elite Eco 20 (or Kelty Cosmic 20 Synthetic)</t>
         </is>
       </c>
       <c r="D5" s="33" t="n">
         <v>53</v>
       </c>
       <c r="E5" s="34" t="n">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
@@ -6119,7 +6119,7 @@
         <v>26</v>
       </c>
       <c r="N5" s="34" t="n">
-        <v>355</v>
+        <v>280</v>
       </c>
       <c r="O5" s="11" t="inlineStr">
         <is>
@@ -6202,14 +6202,14 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>Insulated Static V (or Static V2)</t>
+          <t>Insulated Static V Peak</t>
         </is>
       </c>
       <c r="D6" s="33" t="n">
         <v>25</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>74.95</v>
+        <v>99.95</v>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
@@ -6338,7 +6338,7 @@
         <v>2</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
@@ -6377,7 +6377,7 @@
         <v>2.5</v>
       </c>
       <c r="N7" s="34" t="n">
-        <v>54.95</v>
+        <v>64.95</v>
       </c>
       <c r="O7" s="11" t="inlineStr">
         <is>
@@ -6416,7 +6416,7 @@
         <v>2.5</v>
       </c>
       <c r="W7" s="34" t="n">
-        <v>54.95</v>
+        <v>59.95</v>
       </c>
       <c r="X7" s="11" t="inlineStr">
         <is>
@@ -6467,7 +6467,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
@@ -6506,7 +6506,7 @@
         <v>5</v>
       </c>
       <c r="N8" s="34" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
@@ -6545,7 +6545,7 @@
         <v>3.5</v>
       </c>
       <c r="W8" s="34" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="X8" s="11" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
@@ -6628,14 +6628,14 @@
       </c>
       <c r="L9" s="35" t="inlineStr">
         <is>
-          <t>Ultra-Sil Dry Sack (set of 2-3 sizes, e.g. 8L + 13L)</t>
+          <t>Ultra-Sil Dry Bag - Set of 3</t>
         </is>
       </c>
       <c r="M9" s="33" t="n">
         <v>2.5</v>
       </c>
       <c r="N9" s="34" t="n">
-        <v>40</v>
+        <v>69.95</v>
       </c>
       <c r="O9" s="11" t="inlineStr">
         <is>
@@ -6674,7 +6674,7 @@
         <v>1</v>
       </c>
       <c r="W9" s="34" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="X9" s="11" t="inlineStr">
         <is>
@@ -6725,7 +6725,7 @@
         <v>1.4</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
         <v>0.9</v>
       </c>
       <c r="N10" s="34" t="n">
-        <v>6</v>
+        <v>2.49</v>
       </c>
       <c r="O10" s="11" t="inlineStr">
         <is>
@@ -6796,7 +6796,7 @@
       </c>
       <c r="U10" s="36" t="inlineStr">
         <is>
-          <t>eVent Dry Pack Liner</t>
+          <t>Evac Lightweight Dry Bag (35L)</t>
         </is>
       </c>
       <c r="V10" s="33" t="n">
@@ -6893,7 +6893,7 @@
         <v>3.5</v>
       </c>
       <c r="N11" s="34" t="n">
-        <v>64.95</v>
+        <v>69.95</v>
       </c>
       <c r="O11" s="11" t="inlineStr">
         <is>
@@ -6932,7 +6932,7 @@
         <v>7.1</v>
       </c>
       <c r="W11" s="34" t="n">
-        <v>154.95</v>
+        <v>131</v>
       </c>
       <c r="X11" s="11" t="inlineStr">
         <is>
@@ -6976,14 +6976,14 @@
       </c>
       <c r="C12" s="32" t="inlineStr">
         <is>
-          <t>Aluminum camp pot ~1.5qt</t>
+          <t>A004-025001 Aluminum Sauce Pan, 1-Quart</t>
         </is>
       </c>
       <c r="D12" s="33" t="n">
         <v>6</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
@@ -7015,14 +7015,14 @@
       </c>
       <c r="L12" s="35" t="inlineStr">
         <is>
-          <t>750ml Titanium Pot (POT-750-RS)</t>
+          <t>750ml Titanium Pot with Bail Handle (POT-750-BH)</t>
         </is>
       </c>
       <c r="M12" s="33" t="n">
         <v>4.1</v>
       </c>
       <c r="N12" s="34" t="n">
-        <v>33.95</v>
+        <v>30</v>
       </c>
       <c r="O12" s="11" t="inlineStr">
         <is>
@@ -7054,18 +7054,18 @@
       </c>
       <c r="U12" s="36" t="inlineStr">
         <is>
-          <t>Titanium UL Pasta Pot (ECA267)</t>
+          <t>Trek 900 Titanium Cookset</t>
         </is>
       </c>
       <c r="V12" s="33" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="W12" s="34" t="n">
-        <v>54.99</v>
+        <v>54.95</v>
       </c>
       <c r="X12" s="11" t="inlineStr">
         <is>
-          <t>$35-45 (limited US stock)</t>
+          <t>$35-45</t>
         </is>
       </c>
       <c r="Y12" s="11" t="n">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="AA12" s="11" t="inlineStr">
         <is>
-          <t>Long-time favorite among serious UL hikers for its insulated handles and slightly better pour spout; Treeline Review calls it a runner-up 'Best Upgrade' pick, but flags Evernew has cut back US distribution, making it harder to buy than TOAKS in 2026.</t>
+          <t>Snow Peak's Trek 900 is the standard premium alternative once Evernew stock dries up; Treeline Review and forum threads treat TOAKS/Snow Peak/Evernew as near-interchangeable in quality at this size.</t>
         </is>
       </c>
       <c r="AB12" s="11" t="inlineStr">
@@ -7105,11 +7105,11 @@
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>PowerMax 100g canister</t>
+          <t>Butane/Propane Mix Fuel, 7.75oz (220g)</t>
         </is>
       </c>
       <c r="D13" s="33" t="n">
-        <v>7.4</v>
+        <v>7.75</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>5.97</v>
@@ -7151,7 +7151,7 @@
         <v>13.7</v>
       </c>
       <c r="N13" s="34" t="n">
-        <v>10.95</v>
+        <v>6.95</v>
       </c>
       <c r="O13" s="11" t="inlineStr">
         <is>
@@ -7190,7 +7190,7 @@
         <v>7.6</v>
       </c>
       <c r="W13" s="34" t="n">
-        <v>6.95</v>
+        <v>5.95</v>
       </c>
       <c r="X13" s="11" t="inlineStr">
         <is>
@@ -7234,14 +7234,14 @@
       </c>
       <c r="C14" s="32" t="inlineStr">
         <is>
-          <t>Titanium long-handled spork</t>
+          <t>Titanium Spork</t>
         </is>
       </c>
       <c r="D14" s="33" t="n">
         <v>0.6</v>
       </c>
       <c r="E14" s="34" t="n">
-        <v>7.99</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
@@ -7273,14 +7273,14 @@
       </c>
       <c r="L14" s="35" t="inlineStr">
         <is>
-          <t>Alpha Light Long Spoon</t>
+          <t>Frontier Ultralight Spoon - Long Handle</t>
         </is>
       </c>
       <c r="M14" s="33" t="n">
         <v>0.6</v>
       </c>
       <c r="N14" s="34" t="n">
-        <v>9.949999999999999</v>
+        <v>10.95</v>
       </c>
       <c r="O14" s="11" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         <v>0.6</v>
       </c>
       <c r="W14" s="34" t="n">
-        <v>14.5</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="X14" s="11" t="inlineStr">
         <is>
@@ -7370,7 +7370,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="34" t="n">
-        <v>29.96</v>
+        <v>45.95</v>
       </c>
       <c r="F15" s="11" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
         <v>15.9</v>
       </c>
       <c r="W15" s="34" t="n">
-        <v>89.95</v>
+        <v>99.95</v>
       </c>
       <c r="X15" s="11" t="inlineStr">
         <is>
@@ -7499,7 +7499,7 @@
         <v>1.6</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
@@ -7538,7 +7538,7 @@
         <v>1.4</v>
       </c>
       <c r="N16" s="34" t="n">
-        <v>21.95</v>
+        <v>18</v>
       </c>
       <c r="O16" s="11" t="inlineStr">
         <is>
@@ -7577,7 +7577,7 @@
         <v>3.6</v>
       </c>
       <c r="W16" s="34" t="n">
-        <v>27.95</v>
+        <v>25</v>
       </c>
       <c r="X16" s="11" t="inlineStr">
         <is>
@@ -7621,14 +7621,14 @@
       </c>
       <c r="C17" s="32" t="inlineStr">
         <is>
-          <t>PCT-style bear hang kit (rope + stuff sack + carabiner)</t>
+          <t>Easy to Throw Bear Bag Hanging Kit (#371486)</t>
         </is>
       </c>
       <c r="D17" s="33" t="n">
         <v>6</v>
       </c>
       <c r="E17" s="34" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F17" s="11" t="inlineStr">
         <is>
@@ -7667,7 +7667,7 @@
         <v>10.8</v>
       </c>
       <c r="N17" s="34" t="n">
-        <v>109.9</v>
+        <v>149.95</v>
       </c>
       <c r="O17" s="11" t="inlineStr">
         <is>
@@ -7796,7 +7796,7 @@
         <v>3</v>
       </c>
       <c r="N18" s="34" t="n">
-        <v>44.95</v>
+        <v>59.95</v>
       </c>
       <c r="O18" s="11" t="inlineStr">
         <is>
@@ -7879,14 +7879,14 @@
       </c>
       <c r="C19" s="32" t="inlineStr">
         <is>
-          <t>PowerCore Slim 10000</t>
+          <t>Power Bank, 10,000mAh Portable Charger (PowerIQ, USB-C)</t>
         </is>
       </c>
       <c r="D19" s="33" t="n">
         <v>6.3</v>
       </c>
       <c r="E19" s="34" t="n">
-        <v>23.99</v>
+        <v>21.99</v>
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
@@ -7925,7 +7925,7 @@
         <v>5.1</v>
       </c>
       <c r="N19" s="34" t="n">
-        <v>54.95</v>
+        <v>64.95</v>
       </c>
       <c r="O19" s="11" t="inlineStr">
         <is>
@@ -7964,7 +7964,7 @@
         <v>5</v>
       </c>
       <c r="W19" s="34" t="n">
-        <v>59.95</v>
+        <v>83.95</v>
       </c>
       <c r="X19" s="11" t="inlineStr">
         <is>
@@ -8054,7 +8054,7 @@
         <v>5.4</v>
       </c>
       <c r="N20" s="34" t="n">
-        <v>199.99</v>
+        <v>199</v>
       </c>
       <c r="O20" s="11" t="inlineStr">
         <is>
@@ -8273,7 +8273,7 @@
         <v>1.6</v>
       </c>
       <c r="E22" s="34" t="n">
-        <v>19.95</v>
+        <v>22</v>
       </c>
       <c r="F22" s="11" t="inlineStr">
         <is>
@@ -8312,7 +8312,7 @@
         <v>7.2</v>
       </c>
       <c r="N22" s="34" t="n">
-        <v>44.95</v>
+        <v>49.95</v>
       </c>
       <c r="O22" s="11" t="inlineStr">
         <is>
@@ -8441,7 +8441,7 @@
         <v>4.4</v>
       </c>
       <c r="N23" s="34" t="n">
-        <v>31.95</v>
+        <v>44.99</v>
       </c>
       <c r="O23" s="11" t="inlineStr">
         <is>
@@ -8480,7 +8480,7 @@
         <v>16</v>
       </c>
       <c r="W23" s="34" t="n">
-        <v>74.95</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="X23" s="11" t="inlineStr">
         <is>
@@ -8524,14 +8524,14 @@
       </c>
       <c r="C24" s="32" t="inlineStr">
         <is>
-          <t>Plastic trowel + basic hygiene bag</t>
+          <t>Backpackers Trowel + basic hygiene bag</t>
         </is>
       </c>
       <c r="D24" s="33" t="n">
         <v>2</v>
       </c>
       <c r="E24" s="34" t="n">
-        <v>8</v>
+        <v>8.75</v>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
@@ -8570,7 +8570,7 @@
         <v>2.4</v>
       </c>
       <c r="N24" s="34" t="n">
-        <v>9.949999999999999</v>
+        <v>7.95</v>
       </c>
       <c r="O24" s="11" t="inlineStr">
         <is>
@@ -8602,14 +8602,14 @@
       </c>
       <c r="U24" s="36" t="inlineStr">
         <is>
-          <t>The Deuce of Spades #2 (titanium)</t>
+          <t>The DirtSaw Deuce #2 Trowel</t>
         </is>
       </c>
       <c r="V24" s="33" t="n">
         <v>0.6</v>
       </c>
       <c r="W24" s="34" t="n">
-        <v>24.95</v>
+        <v>21.95</v>
       </c>
       <c r="X24" s="11" t="inlineStr">
         <is>
@@ -8660,7 +8660,7 @@
         <v>18</v>
       </c>
       <c r="E25" s="34" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
@@ -8738,7 +8738,7 @@
         <v>10.9</v>
       </c>
       <c r="W25" s="34" t="n">
-        <v>189.95</v>
+        <v>219.95</v>
       </c>
       <c r="X25" s="11" t="inlineStr">
         <is>
@@ -8911,14 +8911,14 @@
       </c>
       <c r="C27" s="32" t="inlineStr">
         <is>
-          <t>Foam slide sandals</t>
+          <t>Gabe Cloud Slide Sandals</t>
         </is>
       </c>
       <c r="D27" s="33" t="n">
         <v>6</v>
       </c>
       <c r="E27" s="34" t="n">
-        <v>9.99</v>
+        <v>19.99</v>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
@@ -8989,14 +8989,14 @@
       </c>
       <c r="U27" s="36" t="inlineStr">
         <is>
-          <t>Z-Trail sandal</t>
+          <t>Z-Trail EV Sandals</t>
         </is>
       </c>
       <c r="V27" s="33" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="W27" s="34" t="n">
-        <v>69.98999999999999</v>
+        <v>80</v>
       </c>
       <c r="X27" s="11" t="inlineStr">
         <is>
@@ -9055,11 +9055,11 @@
         </is>
       </c>
       <c r="G28" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>Fine for warm-ish days (50s-60s) with wool socks; cold nights mean you must have a fully dry pair to change into</t>
+          <t>BEGINNER CAUTION: fine for warm-ish days (50s-60s) with wool socks, but repeated wading in low-30s/40s creek water in non-insulated mesh trail runners risks cold feet/mild hypothermia for someone inexperienced with cold-water wading; a beginner should plan on wading boots/neoprene socks or accept wet feet only briefly and dry out fast near a fire, not as an all-day creek-panning shoe</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -9254,7 +9254,7 @@
         <v>3.2</v>
       </c>
       <c r="W29" s="34" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="X29" s="11" t="inlineStr">
         <is>
@@ -9512,7 +9512,7 @@
         <v>8.9</v>
       </c>
       <c r="W31" s="34" t="n">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="X31" s="11" t="inlineStr">
         <is>
@@ -9563,7 +9563,7 @@
         <v>12</v>
       </c>
       <c r="E32" s="34" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
@@ -9692,7 +9692,7 @@
         <v>8</v>
       </c>
       <c r="E33" s="34" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
@@ -9770,7 +9770,7 @@
         <v>11</v>
       </c>
       <c r="W33" s="34" t="n">
-        <v>190</v>
+        <v>235</v>
       </c>
       <c r="X33" s="11" t="inlineStr">
         <is>
@@ -9821,7 +9821,7 @@
         <v>11</v>
       </c>
       <c r="E34" s="34" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="F34" s="11" t="inlineStr">
         <is>
@@ -9892,14 +9892,14 @@
       </c>
       <c r="U34" s="36" t="inlineStr">
         <is>
-          <t>Stretch Zion Cargo Pants</t>
+          <t>Stretch Zion Straight Pants (cargo version discontinued, replaced by current lineup)</t>
         </is>
       </c>
       <c r="V34" s="33" t="n">
         <v>14</v>
       </c>
       <c r="W34" s="34" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="X34" s="11" t="inlineStr">
         <is>
@@ -10408,7 +10408,7 @@
       </c>
       <c r="U38" s="36" t="inlineStr">
         <is>
-          <t>Cairn Adventure Sandals</t>
+          <t>Cairn Evo Adventure Sandals (current lineup; original Cairn Adventure Sandal discontinued)</t>
         </is>
       </c>
       <c r="V38" s="33" t="n">
@@ -10802,7 +10802,7 @@
         <v>38</v>
       </c>
       <c r="W41" s="34" t="n">
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="X41" s="11" t="inlineStr">
         <is>
@@ -11627,7 +11627,7 @@
         <v>1</v>
       </c>
       <c r="E48" s="34" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F48" s="11" t="inlineStr">
         <is>
@@ -11705,7 +11705,7 @@
         <v>2</v>
       </c>
       <c r="W48" s="34" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="X48" s="11" t="inlineStr">
         <is>
@@ -11756,7 +11756,7 @@
         <v>6</v>
       </c>
       <c r="E49" s="34" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
@@ -11795,7 +11795,7 @@
         <v>0.6</v>
       </c>
       <c r="N49" s="34" t="n">
-        <v>22.5</v>
+        <v>20.95</v>
       </c>
       <c r="O49" s="11" t="inlineStr">
         <is>
@@ -12131,7 +12131,7 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>30F-rated sleeping bag/quilt (RECOMMENDED default)</t>
+          <t>30F-rated sleeping bag/quilt (RECOMMENDED default -- beginner-safe pick)</t>
         </is>
       </c>
       <c r="C52" s="32" t="inlineStr">
@@ -12415,7 +12415,7 @@
       </c>
       <c r="E2" s="37" t="inlineStr">
         <is>
-          <t>Rook 50 (men's) / Renn 50 (women's)</t>
+          <t>Rook 65 (men's) / Renn 65 (women's)</t>
         </is>
       </c>
       <c r="F2" s="39" t="n">
@@ -12427,11 +12427,11 @@
         </is>
       </c>
       <c r="H2" s="40" t="n">
-        <v>155</v>
+        <v>205</v>
       </c>
       <c r="I2" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/231462/osprey-rook-50-pack-mens</t>
+          <t>https://www.rei.com/product/231463/osprey-rook-65-pack-mens</t>
         </is>
       </c>
       <c r="J2" s="38" t="inlineStr">
@@ -12706,11 +12706,11 @@
         </is>
       </c>
       <c r="H5" s="40" t="n">
-        <v>159</v>
+        <v>259</v>
       </c>
       <c r="I5" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/199426/rei-co-op-trail-hut-2-tent</t>
+          <t>https://www.rei.com/product/C03309/rei-co-op-trail-hut-2-tent-with-footprint</t>
         </is>
       </c>
       <c r="J5" s="38" t="inlineStr">
@@ -12892,7 +12892,7 @@
         </is>
       </c>
       <c r="H7" s="40" t="n">
-        <v>699</v>
+        <v>749</v>
       </c>
       <c r="I7" s="41" t="inlineStr">
         <is>
@@ -12973,7 +12973,7 @@
       </c>
       <c r="E8" s="37" t="inlineStr">
         <is>
-          <t>Trestles 15 (or Kelty Cosmic 20 Synthetic)</t>
+          <t>Trestles Elite Eco 20 (or Kelty Cosmic 20 Synthetic)</t>
         </is>
       </c>
       <c r="F8" s="39" t="n">
@@ -12985,11 +12985,11 @@
         </is>
       </c>
       <c r="H8" s="40" t="n">
-        <v>99</v>
+        <v>179</v>
       </c>
       <c r="I8" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/126630/marmot-trestles-15-sleeping-bag</t>
+          <t>https://www.rei.com/product/245787/marmot-trestles-elite-eco-20-sleeping-bag</t>
         </is>
       </c>
       <c r="J8" s="38" t="inlineStr">
@@ -13078,7 +13078,7 @@
         </is>
       </c>
       <c r="H9" s="40" t="n">
-        <v>355</v>
+        <v>280</v>
       </c>
       <c r="I9" s="41" t="inlineStr">
         <is>
@@ -13252,7 +13252,7 @@
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
-          <t>Insulated Static V (or Static V2)</t>
+          <t>Insulated Static V Peak</t>
         </is>
       </c>
       <c r="F11" s="39" t="n">
@@ -13264,11 +13264,11 @@
         </is>
       </c>
       <c r="H11" s="40" t="n">
-        <v>74.95</v>
+        <v>99.95</v>
       </c>
       <c r="I11" s="41" t="inlineStr">
         <is>
-          <t>https://klymit.com/products/insulated-static-v-sleeping-pad-4-pack</t>
+          <t>https://klymit.com/products/insulated-static-v-peak-sleeping-pads</t>
         </is>
       </c>
       <c r="J11" s="38" t="inlineStr">
@@ -13543,11 +13543,11 @@
         </is>
       </c>
       <c r="H14" s="40" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I14" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/199426/rei-co-op-trail-hut-2-tent</t>
+          <t>https://www.amazon.com/dp/B0896WCB5D</t>
         </is>
       </c>
       <c r="J14" s="38" t="inlineStr">
@@ -13636,7 +13636,7 @@
         </is>
       </c>
       <c r="H15" s="40" t="n">
-        <v>54.95</v>
+        <v>64.95</v>
       </c>
       <c r="I15" s="41" t="inlineStr">
         <is>
@@ -13686,7 +13686,7 @@
       </c>
       <c r="S15" s="38" t="inlineStr">
         <is>
-          <t>The standard (non-down) Aeros Premium is ~$10 cheaper and works fine too if warmth-at-the-head doesn't matter</t>
+          <t>The standard (non-down) Aeros Premium is ~$10 cheaper and works fine too if warmth-at-the-head doesn't matter | TIER ODDITY: Value ($64.95) costs more than Premium ($59.95) in this category -- kept as sourced, not auto-corrected.</t>
         </is>
       </c>
       <c r="T15">
@@ -13729,11 +13729,11 @@
         </is>
       </c>
       <c r="H16" s="40" t="n">
-        <v>54.95</v>
+        <v>59.95</v>
       </c>
       <c r="I16" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/128558/nemo-fillo-elite-pillow</t>
+          <t>https://www.rei.com/product/170457/nemo-fillo-elite-pillow</t>
         </is>
       </c>
       <c r="J16" s="38" t="inlineStr">
@@ -13779,7 +13779,7 @@
       </c>
       <c r="S16" s="38" t="inlineStr">
         <is>
-          <t>Genuinely a coin-flip vs. the Sea to Summit Aeros — 'premium' here reflects feel/comfort preference, not a real capability gap; buy whichever is on sale</t>
+          <t>Genuinely a coin-flip vs. the Sea to Summit Aeros — 'premium' here reflects feel/comfort preference, not a real capability gap; buy whichever is on sale | TIER ODDITY: Premium ($59.95) is cheaper than Value ($64.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T16">
@@ -13822,11 +13822,11 @@
         </is>
       </c>
       <c r="H17" s="40" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I17" s="41" t="inlineStr">
         <is>
-          <t>https://www.gossamergear.com/products/polycryo-ground-cloth</t>
+          <t>https://www.gossamergear.com/products/polycryo-tent-footprint-ground-cloths</t>
         </is>
       </c>
       <c r="J17" s="38" t="inlineStr">
@@ -13915,11 +13915,11 @@
         </is>
       </c>
       <c r="H18" s="40" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I18" s="41" t="inlineStr">
         <is>
-          <t>https://sectionhiker.com/ultralight-backpacking-tent-footprint-substitutions/</t>
+          <t>https://www.amazon.com/dp/B0CWDQDS32</t>
         </is>
       </c>
       <c r="J18" s="38" t="inlineStr">
@@ -14008,11 +14008,11 @@
         </is>
       </c>
       <c r="H19" s="40" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="I19" s="41" t="inlineStr">
         <is>
-          <t>https://durstongear.com/products/x-mid-2-footprint</t>
+          <t>https://durstongear.com/products/x-mid-2-groundsheet</t>
         </is>
       </c>
       <c r="J19" s="38" t="inlineStr">
@@ -14101,11 +14101,11 @@
         </is>
       </c>
       <c r="H20" s="40" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="I20" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/55048225</t>
+          <t>https://www.amazon.com/dp/B0028CXKQE</t>
         </is>
       </c>
       <c r="J20" s="38" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="E21" s="37" t="inlineStr">
         <is>
-          <t>Ultra-Sil Dry Sack (set of 2-3 sizes, e.g. 8L + 13L)</t>
+          <t>Ultra-Sil Dry Bag - Set of 3</t>
         </is>
       </c>
       <c r="F21" s="39" t="n">
@@ -14194,11 +14194,11 @@
         </is>
       </c>
       <c r="H21" s="40" t="n">
-        <v>40</v>
+        <v>69.95</v>
       </c>
       <c r="I21" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/205635/sea-to-summit-ultra-sil-dry-sack-set-of-3</t>
+          <t>https://www.rei.com/product/218733/sea-to-summit-ultra-sil-dry-bag-set-of-3</t>
         </is>
       </c>
       <c r="J21" s="38" t="inlineStr">
@@ -14244,7 +14244,7 @@
       </c>
       <c r="S21" s="38" t="inlineStr">
         <is>
-          <t>Sized an 8L for the sleeping bag/quilt + a 4L or 1L for electronics/fire-starting kit covers this trip well | TIER ODDITY: Value ($40.00) costs more than Premium ($33.00) in this category -- kept as sourced, not auto-corrected.</t>
+          <t>Sized an 8L for the sleeping bag/quilt + a 4L or 1L for electronics/fire-starting kit covers this trip well | TIER ODDITY: Value ($69.95) costs more than Premium ($31.00) in this category -- kept as sourced, not auto-corrected.</t>
         </is>
       </c>
       <c r="T21">
@@ -14287,11 +14287,11 @@
         </is>
       </c>
       <c r="H22" s="40" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I22" s="41" t="inlineStr">
         <is>
-          <t>https://hyperlitemountaingear.com/products/stuff-sacks</t>
+          <t>https://hyperlitemountaingear.com/products/drawstring-stuff-sacks</t>
         </is>
       </c>
       <c r="J22" s="38" t="inlineStr">
@@ -14337,7 +14337,7 @@
       </c>
       <c r="S22" s="38" t="inlineStr">
         <is>
-          <t>Skip for this trip specifically — recommended only if the buyer is already committed to backpacking as an ongoing hobby | TIER ODDITY: Premium ($33.00) is cheaper than Value ($40.00) in this category -- kept as sourced.</t>
+          <t>Skip for this trip specifically — recommended only if the buyer is already committed to backpacking as an ongoing hobby | TIER ODDITY: Premium ($31.00) is cheaper than Value ($69.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T22">
@@ -14380,11 +14380,11 @@
         </is>
       </c>
       <c r="H23" s="40" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I23" s="41" t="inlineStr">
         <is>
-          <t>https://www.99boulders.com/best-pack-liners</t>
+          <t>https://www.amazon.com/dp/B07SM88VVF</t>
         </is>
       </c>
       <c r="J23" s="38" t="inlineStr">
@@ -14430,7 +14430,7 @@
       </c>
       <c r="S23" s="38" t="inlineStr">
         <is>
-          <t>Already correctly identified in the existing gear.md as the go-to; this confirms it against wider community sourcing</t>
+          <t>Already correctly identified in the existing gear.md as the go-to; this confirms it against wider community sourcing | TIER ODDITY: Budget ($10.00) costs more than Value ($2.49) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T23">
@@ -14473,7 +14473,7 @@
         </is>
       </c>
       <c r="H24" s="40" t="n">
-        <v>6</v>
+        <v>2.49</v>
       </c>
       <c r="I24" s="41" t="inlineStr">
         <is>
@@ -14523,7 +14523,7 @@
       </c>
       <c r="S24" s="38" t="inlineStr">
         <is>
-          <t>Marginal upgrade — not worth agonizing over vs. the free compactor-bag option for a single trip</t>
+          <t>Marginal upgrade — not worth agonizing over vs. the free compactor-bag option for a single trip | TIER ODDITY: Value ($2.49) is cheaper than Budget ($10.00) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T24">
@@ -14554,7 +14554,7 @@
       </c>
       <c r="E25" s="37" t="inlineStr">
         <is>
-          <t>eVent Dry Pack Liner</t>
+          <t>Evac Lightweight Dry Bag (35L)</t>
         </is>
       </c>
       <c r="F25" s="39" t="n">
@@ -14570,7 +14570,7 @@
       </c>
       <c r="I25" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/106325/sea-to-summit-event-dry-pack-liner</t>
+          <t>https://www.rei.com/product/246133/sea-to-summit-evac-lightweight-dry-bag</t>
         </is>
       </c>
       <c r="J25" s="38" t="inlineStr">
@@ -14752,11 +14752,11 @@
         </is>
       </c>
       <c r="H27" s="40" t="n">
-        <v>64.95</v>
+        <v>69.95</v>
       </c>
       <c r="I27" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/128793/soto-windmaster-stove</t>
+          <t>https://www.rei.com/product/177954/soto-windmaster-stove-with-4flex-pot-support</t>
         </is>
       </c>
       <c r="J27" s="38" t="inlineStr">
@@ -14845,11 +14845,11 @@
         </is>
       </c>
       <c r="H28" s="40" t="n">
-        <v>154.95</v>
+        <v>131</v>
       </c>
       <c r="I28" s="41" t="inlineStr">
         <is>
-          <t>https://www.jetboil.com/products/stash-cooking-system</t>
+          <t>https://www.amazon.com/Jetboil-Ultralight-Camping-Backpacking-Cooking/dp/B08QRLT8QH</t>
         </is>
       </c>
       <c r="J28" s="38" t="inlineStr">
@@ -14921,12 +14921,12 @@
       </c>
       <c r="D29" s="37" t="inlineStr">
         <is>
-          <t>IMUSA / generic</t>
+          <t>IMUSA</t>
         </is>
       </c>
       <c r="E29" s="37" t="inlineStr">
         <is>
-          <t>Aluminum camp pot ~1.5qt</t>
+          <t>A004-025001 Aluminum Sauce Pan, 1-Quart</t>
         </is>
       </c>
       <c r="F29" s="39" t="n">
@@ -14934,15 +14934,15 @@
       </c>
       <c r="G29" s="38" t="inlineStr">
         <is>
-          <t>typical stamped-aluminum camp pot weight; EST from category norms, not individually spec-verified this session</t>
+          <t>typical stamped-aluminum camp pot weight; EST from category norms, not individually spec-verified this session; only 1qt capacity — buy two for group boiling of 6</t>
         </is>
       </c>
       <c r="H29" s="40" t="n">
-        <v>11.99</v>
+        <v>12.99</v>
       </c>
       <c r="I29" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/browse/camping-cookware</t>
+          <t>https://www.amazon.com/IMUSA-A004-025001-Aluminum-1-Quart-Silver/dp/B0018E9UV2</t>
         </is>
       </c>
       <c r="J29" s="38" t="inlineStr">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="E30" s="37" t="inlineStr">
         <is>
-          <t>750ml Titanium Pot (POT-750-RS)</t>
+          <t>750ml Titanium Pot with Bail Handle (POT-750-BH)</t>
         </is>
       </c>
       <c r="F30" s="39" t="n">
@@ -15031,7 +15031,7 @@
         </is>
       </c>
       <c r="H30" s="40" t="n">
-        <v>33.95</v>
+        <v>30</v>
       </c>
       <c r="I30" s="41" t="inlineStr">
         <is>
@@ -15107,43 +15107,43 @@
       </c>
       <c r="D31" s="37" t="inlineStr">
         <is>
-          <t>Evernew</t>
+          <t>Snow Peak</t>
         </is>
       </c>
       <c r="E31" s="37" t="inlineStr">
         <is>
-          <t>Titanium UL Pasta Pot (ECA267)</t>
+          <t>Trek 900 Titanium Cookset</t>
         </is>
       </c>
       <c r="F31" s="39" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="G31" s="38" t="inlineStr">
         <is>
-          <t>manufacturer spec ~100g/3.5oz for the 0.9L pasta pot; increasingly hard to find due to reduced US distribution</t>
+          <t>REI spec 6oz/170g for the 2-piece cookset (900ml pot + pan/lid); swapped in for the Evernew pasta pot, which is discontinued/unavailable in the US as of 2026</t>
         </is>
       </c>
       <c r="H31" s="40" t="n">
-        <v>54.99</v>
+        <v>54.95</v>
       </c>
       <c r="I31" s="41" t="inlineStr">
         <is>
-          <t>https://www.evernew-outdoor.jp/</t>
+          <t>https://www.rei.com/product/768602/snow-peak-trek-900-titanium-cookset</t>
         </is>
       </c>
       <c r="J31" s="38" t="inlineStr">
         <is>
-          <t>$35-45 (limited US stock)</t>
+          <t>$35-45</t>
         </is>
       </c>
       <c r="K31" s="38" t="inlineStr">
         <is>
-          <t>Evernew Japan direct, occasional REI/Backcountry stock, eBay</t>
+          <t>REI, Amazon, Snow Peak direct</t>
         </is>
       </c>
       <c r="L31" s="38" t="inlineStr">
         <is>
-          <t>Long-time favorite among serious UL hikers for its insulated handles and slightly better pour spout; Treeline Review calls it a runner-up 'Best Upgrade' pick, but flags Evernew has cut back US distribution, making it harder to buy than TOAKS in 2026.</t>
+          <t>Snow Peak's Trek 900 is the standard premium alternative once Evernew stock dries up; Treeline Review and forum threads treat TOAKS/Snow Peak/Evernew as near-interchangeable in quality at this size.</t>
         </is>
       </c>
       <c r="M31" s="38" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="S31" s="38" t="inlineStr">
         <is>
-          <t>Group share $9.17 — flag as possibly discontinued/limited in US retail as of 2026</t>
+          <t>Group share $9.16</t>
         </is>
       </c>
       <c r="T31">
@@ -15205,15 +15205,15 @@
       </c>
       <c r="E32" s="37" t="inlineStr">
         <is>
-          <t>PowerMax 100g canister</t>
+          <t>Butane/Propane Mix Fuel, 7.75oz (220g)</t>
         </is>
       </c>
       <c r="F32" s="39" t="n">
-        <v>7.4</v>
+        <v>7.75</v>
       </c>
       <c r="G32" s="38" t="inlineStr">
         <is>
-          <t>100g fuel + canister, ~7.4oz total per typical 100g canister spec</t>
+          <t>Walmart spec, 220g fuel canister</t>
         </is>
       </c>
       <c r="H32" s="40" t="n">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="I32" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/browse/camping-fuel</t>
+          <t>https://www.walmart.com/ip/Coleman-Butane-Propane-Mix-Fuel-7-75oz/20595064</t>
         </is>
       </c>
       <c r="J32" s="38" t="inlineStr">
@@ -15310,7 +15310,7 @@
         </is>
       </c>
       <c r="H33" s="40" t="n">
-        <v>10.95</v>
+        <v>6.95</v>
       </c>
       <c r="I33" s="41" t="inlineStr">
         <is>
@@ -15360,7 +15360,7 @@
       </c>
       <c r="S33" s="38" t="inlineStr">
         <is>
-          <t>Group share $1.83; consider the 4oz can instead ($6-7) to match actual need | TIER ODDITY: Value ($10.95) costs more than Premium ($6.95) in this category -- kept as sourced, not auto-corrected.</t>
+          <t>Group share $1.83; consider the 4oz can instead ($6-7) to match actual need | TIER ODDITY: Value ($6.95) costs more than Premium ($5.95) in this category -- kept as sourced, not auto-corrected.</t>
         </is>
       </c>
       <c r="T33">
@@ -15403,11 +15403,11 @@
         </is>
       </c>
       <c r="H34" s="40" t="n">
-        <v>6.95</v>
+        <v>5.95</v>
       </c>
       <c r="I34" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/807823/msr-isopro-fuel</t>
+          <t>https://www.rei.com/product/849634/msr-isopro-fuel-canister-39-oz-110-g</t>
         </is>
       </c>
       <c r="J34" s="38" t="inlineStr">
@@ -15453,7 +15453,7 @@
       </c>
       <c r="S34" s="38" t="inlineStr">
         <is>
-          <t>Group share $1.16; fuel is not a category worth upgrading — put the money into the stove instead | TIER ODDITY: Premium ($6.95) is cheaper than Value ($10.95) in this category -- kept as sourced.</t>
+          <t>Group share $1.16; fuel is not a category worth upgrading — put the money into the stove instead | TIER ODDITY: Premium ($5.95) is cheaper than Value ($6.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T34">
@@ -15479,12 +15479,12 @@
       </c>
       <c r="D35" s="37" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>TOAKS</t>
         </is>
       </c>
       <c r="E35" s="37" t="inlineStr">
         <is>
-          <t>Titanium long-handled spork</t>
+          <t>Titanium Spork</t>
         </is>
       </c>
       <c r="F35" s="39" t="n">
@@ -15496,11 +15496,11 @@
         </is>
       </c>
       <c r="H35" s="40" t="n">
-        <v>7.99</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="I35" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/s?k=titanium+long+spork</t>
+          <t>https://www.rei.com/product/139476/toaks-titanium-spork</t>
         </is>
       </c>
       <c r="J35" s="38" t="inlineStr">
@@ -15577,7 +15577,7 @@
       </c>
       <c r="E36" s="37" t="inlineStr">
         <is>
-          <t>Alpha Light Long Spoon</t>
+          <t>Frontier Ultralight Spoon - Long Handle</t>
         </is>
       </c>
       <c r="F36" s="39" t="n">
@@ -15589,7 +15589,7 @@
         </is>
       </c>
       <c r="H36" s="40" t="n">
-        <v>9.949999999999999</v>
+        <v>10.95</v>
       </c>
       <c r="I36" s="41" t="inlineStr">
         <is>
@@ -15637,7 +15637,11 @@
       <c r="R36" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S36" s="38" t="inlineStr"/>
+      <c r="S36" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($10.95) costs more than Premium ($9.95) in this category -- kept as sourced, not auto-corrected.</t>
+        </is>
+      </c>
       <c r="T36">
         <f>A36&amp;"|"&amp;C36</f>
         <v/>
@@ -15678,11 +15682,11 @@
         </is>
       </c>
       <c r="H37" s="40" t="n">
-        <v>14.5</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="I37" s="41" t="inlineStr">
         <is>
-          <t>https://www.snowpeak.com/products/spork-single-eat-105</t>
+          <t>https://www.rei.com/product/660002/snow-peak-titanium-spork</t>
         </is>
       </c>
       <c r="J37" s="38" t="inlineStr">
@@ -15728,7 +15732,7 @@
       </c>
       <c r="S37" s="38" t="inlineStr">
         <is>
-          <t>Skip this upgrade — put the money toward the water filter or bag instead</t>
+          <t>Skip this upgrade — put the money toward the water filter or bag instead | TIER ODDITY: Premium ($9.95) is cheaper than Value ($10.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T37">
@@ -15771,11 +15775,11 @@
         </is>
       </c>
       <c r="H38" s="40" t="n">
-        <v>29.96</v>
+        <v>45.95</v>
       </c>
       <c r="I38" s="41" t="inlineStr">
         <is>
-          <t>https://www.sawyer.com/products/squeeze-filter</t>
+          <t>https://www.rei.com/product/103050/sawyer-squeeze-water-filter-system</t>
         </is>
       </c>
       <c r="J38" s="38" t="inlineStr">
@@ -15821,7 +15825,7 @@
       </c>
       <c r="S38" s="38" t="inlineStr">
         <is>
-          <t>Group share $5.00</t>
+          <t>Group share $5.00 | TIER ODDITY: Budget ($45.95) costs more than Value ($44.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T38">
@@ -15914,7 +15918,7 @@
       </c>
       <c r="S39" s="38" t="inlineStr">
         <is>
-          <t>Group share $7.49; still needs to sleep in the bag on the cold night</t>
+          <t>Group share $7.49; still needs to sleep in the bag on the cold night | TIER ODDITY: Value ($44.95) is cheaper than Budget ($45.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T39">
@@ -15957,11 +15961,11 @@
         </is>
       </c>
       <c r="H40" s="40" t="n">
-        <v>89.95</v>
+        <v>99.95</v>
       </c>
       <c r="I40" s="41" t="inlineStr">
         <is>
-          <t>https://grayl.com/products/geopress</t>
+          <t>https://www.rei.com/product/150116/grayl-geopress-water-filter-and-purifier-bottle-24-fl-oz</t>
         </is>
       </c>
       <c r="J40" s="38" t="inlineStr">
@@ -16050,11 +16054,11 @@
         </is>
       </c>
       <c r="H41" s="40" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="I41" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/smartwater-1-liter/</t>
+          <t>https://www.walmart.com/ip/smartwater-vapor-distilled-premium-water-1-liter-bottle/14944716</t>
         </is>
       </c>
       <c r="J41" s="38" t="inlineStr">
@@ -16143,7 +16147,7 @@
         </is>
       </c>
       <c r="H42" s="40" t="n">
-        <v>21.95</v>
+        <v>18</v>
       </c>
       <c r="I42" s="41" t="inlineStr">
         <is>
@@ -16232,11 +16236,11 @@
         </is>
       </c>
       <c r="H43" s="40" t="n">
-        <v>27.95</v>
+        <v>25</v>
       </c>
       <c r="I43" s="41" t="inlineStr">
         <is>
-          <t>https://cnocoutdoors.com/products/vecto-2l-water-container</t>
+          <t>https://www.amazon.com/Cnoc-Outdoors-Container-Thread-Orange/dp/B07QBQ894L</t>
         </is>
       </c>
       <c r="J43" s="38" t="inlineStr">
@@ -16308,12 +16312,12 @@
       </c>
       <c r="D44" s="37" t="inlineStr">
         <is>
-          <t>DIY</t>
+          <t>Liberty Mountain</t>
         </is>
       </c>
       <c r="E44" s="37" t="inlineStr">
         <is>
-          <t>PCT-style bear hang kit (rope + stuff sack + carabiner)</t>
+          <t>Easy to Throw Bear Bag Hanging Kit (#371486)</t>
         </is>
       </c>
       <c r="F44" s="39" t="n">
@@ -16325,11 +16329,11 @@
         </is>
       </c>
       <c r="H44" s="40" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="I44" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/c/paracord</t>
+          <t>https://www.amazon.com/Liberty-Mountain-371486-Throw-Hanging/dp/B005U5J934</t>
         </is>
       </c>
       <c r="J44" s="38" t="inlineStr">
@@ -16418,7 +16422,7 @@
         </is>
       </c>
       <c r="H45" s="40" t="n">
-        <v>109.9</v>
+        <v>149.95</v>
       </c>
       <c r="I45" s="41" t="inlineStr">
         <is>
@@ -16468,7 +16472,7 @@
       </c>
       <c r="S45" s="38" t="inlineStr">
         <is>
-          <t>Group share $18.32; this is the pick most aligned with what experienced Southeast hikers use | TIER ODDITY: Value ($109.90) costs more than Premium ($99.95) in this category -- kept as sourced, not auto-corrected.</t>
+          <t>Group share $18.32; this is the pick most aligned with what experienced Southeast hikers use | TIER ODDITY: Value ($149.95) costs more than Premium ($99.95) in this category -- kept as sourced, not auto-corrected.</t>
         </is>
       </c>
       <c r="T45">
@@ -16561,7 +16565,7 @@
       </c>
       <c r="S46" s="38" t="inlineStr">
         <is>
-          <t>Group share $16.66; not necessary for this specific trip | TIER ODDITY: Premium ($99.95) is cheaper than Value ($109.90) in this category -- kept as sourced.</t>
+          <t>Group share $16.66; not necessary for this specific trip | TIER ODDITY: Premium ($99.95) is cheaper than Value ($149.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T46">
@@ -16693,7 +16697,7 @@
         </is>
       </c>
       <c r="H48" s="40" t="n">
-        <v>44.95</v>
+        <v>59.95</v>
       </c>
       <c r="I48" s="41" t="inlineStr">
         <is>
@@ -16741,7 +16745,11 @@
       <c r="R48" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S48" s="38" t="inlineStr"/>
+      <c r="S48" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($59.95) costs more than Premium ($54.95) in this category -- kept as sourced, not auto-corrected.</t>
+        </is>
+      </c>
       <c r="T48">
         <f>A48&amp;"|"&amp;C48</f>
         <v/>
@@ -16786,7 +16794,7 @@
       </c>
       <c r="I49" s="41" t="inlineStr">
         <is>
-          <t>https://flashlight.nitecore.com/product/nu25</t>
+          <t>https://www.nitecore.com/product/nu25</t>
         </is>
       </c>
       <c r="J49" s="38" t="inlineStr">
@@ -16832,7 +16840,7 @@
       </c>
       <c r="S49" s="38" t="inlineStr">
         <is>
-          <t>Bring the power bank to recharge it if the trip runs long</t>
+          <t>Bring the power bank to recharge it if the trip runs long | TIER ODDITY: Premium ($54.95) is cheaper than Value ($59.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T49">
@@ -16863,7 +16871,7 @@
       </c>
       <c r="E50" s="37" t="inlineStr">
         <is>
-          <t>PowerCore Slim 10000</t>
+          <t>Power Bank, 10,000mAh Portable Charger (PowerIQ, USB-C)</t>
         </is>
       </c>
       <c r="F50" s="39" t="n">
@@ -16875,11 +16883,11 @@
         </is>
       </c>
       <c r="H50" s="40" t="n">
-        <v>23.99</v>
+        <v>21.99</v>
       </c>
       <c r="I50" s="41" t="inlineStr">
         <is>
-          <t>https://www.anker.com/products/a1229-powercore-slim-10000</t>
+          <t>https://www.amazon.com/Anker-Portable-Charger-PowerIQ-Battery/dp/B0D5CLSMFB</t>
         </is>
       </c>
       <c r="J50" s="38" t="inlineStr">
@@ -16964,11 +16972,11 @@
         </is>
       </c>
       <c r="H51" s="40" t="n">
-        <v>54.95</v>
+        <v>64.95</v>
       </c>
       <c r="I51" s="41" t="inlineStr">
         <is>
-          <t>https://www.nitecore.com/product/nb10000gen3</t>
+          <t>https://www.amazon.com/NITECORE-NB10000-GEN3-Portable-Charger/dp/B0H85CT2GM</t>
         </is>
       </c>
       <c r="J51" s="38" t="inlineStr">
@@ -17053,11 +17061,11 @@
         </is>
       </c>
       <c r="H52" s="40" t="n">
-        <v>59.95</v>
+        <v>83.95</v>
       </c>
       <c r="I52" s="41" t="inlineStr">
         <is>
-          <t>https://flashlight.nitecore.com/product/nb10000-gen4</t>
+          <t>https://www.amazon.com/Nitecore-NB10000-Gen4-Ultralight-Waterproof/dp/B0H61KHJ1X</t>
         </is>
       </c>
       <c r="J52" s="38" t="inlineStr">
@@ -17239,7 +17247,7 @@
         </is>
       </c>
       <c r="H54" s="40" t="n">
-        <v>199.99</v>
+        <v>199</v>
       </c>
       <c r="I54" s="41" t="inlineStr">
         <is>
@@ -17704,11 +17712,11 @@
         </is>
       </c>
       <c r="H59" s="40" t="n">
-        <v>19.95</v>
+        <v>22</v>
       </c>
       <c r="I59" s="41" t="inlineStr">
         <is>
-          <t>https://www.opinel-usa.com/products/no-08-stainless-steel</t>
+          <t>https://www.rei.com/product/884528/opinel-no-8-beechwood-handle-knife</t>
         </is>
       </c>
       <c r="J59" s="38" t="inlineStr">
@@ -17793,7 +17801,7 @@
         </is>
       </c>
       <c r="H60" s="40" t="n">
-        <v>44.95</v>
+        <v>49.95</v>
       </c>
       <c r="I60" s="41" t="inlineStr">
         <is>
@@ -17886,7 +17894,7 @@
       </c>
       <c r="I61" s="41" t="inlineStr">
         <is>
-          <t>https://www.leatherman.com/skeletool-cx-832180.html</t>
+          <t>https://www.rei.com/product/762082/leatherman-skeletool-cx-multi-tool</t>
         </is>
       </c>
       <c r="J61" s="38" t="inlineStr">
@@ -18064,7 +18072,7 @@
         </is>
       </c>
       <c r="H63" s="40" t="n">
-        <v>31.95</v>
+        <v>44.99</v>
       </c>
       <c r="I63" s="41" t="inlineStr">
         <is>
@@ -18157,7 +18165,7 @@
         </is>
       </c>
       <c r="H64" s="40" t="n">
-        <v>74.95</v>
+        <v>86.48999999999999</v>
       </c>
       <c r="I64" s="41" t="inlineStr">
         <is>
@@ -18238,7 +18246,7 @@
       </c>
       <c r="E65" s="37" t="inlineStr">
         <is>
-          <t>Plastic trowel + basic hygiene bag</t>
+          <t>Backpackers Trowel + basic hygiene bag</t>
         </is>
       </c>
       <c r="F65" s="39" t="n">
@@ -18250,11 +18258,11 @@
         </is>
       </c>
       <c r="H65" s="40" t="n">
-        <v>8</v>
+        <v>8.75</v>
       </c>
       <c r="I65" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/c/first-aid</t>
+          <t>https://www.walmart.com/ip/Coghlan-S-Backpackers-Trowel/23233743</t>
         </is>
       </c>
       <c r="J65" s="38" t="inlineStr">
@@ -18298,7 +18306,11 @@
       <c r="R65" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S65" s="38" t="inlineStr"/>
+      <c r="S65" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Budget ($8.75) costs more than Value ($7.95) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T65">
         <f>A65&amp;"|"&amp;C65</f>
         <v/>
@@ -18339,7 +18351,7 @@
         </is>
       </c>
       <c r="H66" s="40" t="n">
-        <v>9.949999999999999</v>
+        <v>7.95</v>
       </c>
       <c r="I66" s="41" t="inlineStr">
         <is>
@@ -18387,7 +18399,11 @@
       <c r="R66" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S66" s="38" t="inlineStr"/>
+      <c r="S66" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($7.95) is cheaper than Budget ($8.75) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T66">
         <f>A66&amp;"|"&amp;C66</f>
         <v/>
@@ -18416,7 +18432,7 @@
       </c>
       <c r="E67" s="37" t="inlineStr">
         <is>
-          <t>The Deuce of Spades #2 (titanium)</t>
+          <t>The DirtSaw Deuce #2 Trowel</t>
         </is>
       </c>
       <c r="F67" s="39" t="n">
@@ -18428,11 +18444,11 @@
         </is>
       </c>
       <c r="H67" s="40" t="n">
-        <v>24.95</v>
+        <v>21.95</v>
       </c>
       <c r="I67" s="41" t="inlineStr">
         <is>
-          <t>https://www.thetentlab.com/collections/the-deuce</t>
+          <t>https://www.rei.com/product/225131/thetentlab-the-dirtsaw-deuce-2-trowel</t>
         </is>
       </c>
       <c r="J67" s="38" t="inlineStr">
@@ -18517,11 +18533,11 @@
         </is>
       </c>
       <c r="H68" s="40" t="n">
-        <v>35.99</v>
+        <v>39.99</v>
       </c>
       <c r="I68" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/s?k=trailbuddy+trekking+poles</t>
+          <t>https://www.amazon.com/dp/B07C46QPTR</t>
         </is>
       </c>
       <c r="J68" s="38" t="inlineStr">
@@ -18695,11 +18711,11 @@
         </is>
       </c>
       <c r="H70" s="40" t="n">
-        <v>189.95</v>
+        <v>219.95</v>
       </c>
       <c r="I70" s="41" t="inlineStr">
         <is>
-          <t>https://www.blackdiamondequipment.com/en_US/distance-carbon-z-trekking-poles-BD1125.html</t>
+          <t>https://www.rei.com/product/246033/black-diamond-distance-carbon-z-trekking-poles-pair</t>
         </is>
       </c>
       <c r="J70" s="38" t="inlineStr">
@@ -18788,7 +18804,7 @@
       </c>
       <c r="I71" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/c/sleeping-pads</t>
+          <t>https://www.amazon.com/Hit-Delights-Backpacking-Insulation-Lightweight/dp/B06XCWC6T9</t>
         </is>
       </c>
       <c r="J71" s="38" t="inlineStr">
@@ -18798,7 +18814,7 @@
       </c>
       <c r="K71" s="38" t="inlineStr">
         <is>
-          <t>scrap from any CCF sleeping pad</t>
+          <t>scrap cut from any CCF sleeping pad (link is a cheap CCF pad to cut from if none on hand, ~$11)</t>
         </is>
       </c>
       <c r="L71" s="38" t="inlineStr">
@@ -19034,12 +19050,12 @@
       </c>
       <c r="D74" s="37" t="inlineStr">
         <is>
-          <t>generic</t>
+          <t>Alpine Swiss</t>
         </is>
       </c>
       <c r="E74" s="37" t="inlineStr">
         <is>
-          <t>Foam slide sandals</t>
+          <t>Gabe Cloud Slide Sandals</t>
         </is>
       </c>
       <c r="F74" s="39" t="n">
@@ -19051,11 +19067,11 @@
         </is>
       </c>
       <c r="H74" s="40" t="n">
-        <v>9.99</v>
+        <v>19.99</v>
       </c>
       <c r="I74" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/browse/shoes</t>
+          <t>https://www.amazon.com/Alpine-Swiss-Sandals-Adjustable-Athletic/dp/B09G4P66R5</t>
         </is>
       </c>
       <c r="J74" s="38" t="inlineStr">
@@ -19221,7 +19237,7 @@
       </c>
       <c r="E76" s="37" t="inlineStr">
         <is>
-          <t>Z-Trail sandal</t>
+          <t>Z-Trail EV Sandals</t>
         </is>
       </c>
       <c r="F76" s="39" t="n">
@@ -19233,11 +19249,11 @@
         </is>
       </c>
       <c r="H76" s="40" t="n">
-        <v>69.98999999999999</v>
+        <v>80</v>
       </c>
       <c r="I76" s="41" t="inlineStr">
         <is>
-          <t>https://xeroshoes.com/shop/z-trail-mens/</t>
+          <t>https://www.rei.com/product/185226/xero-shoes-z-trail-ev-sandals-mens</t>
         </is>
       </c>
       <c r="J76" s="38" t="inlineStr">
@@ -19361,18 +19377,18 @@
       </c>
       <c r="P77" s="38" t="inlineStr">
         <is>
-          <t>Fine for warm-ish days (50s-60s) with wool socks; cold nights mean you must have a fully dry pair to change into</t>
+          <t>BEGINNER CAUTION: fine for warm-ish days (50s-60s) with wool socks, but repeated wading in low-30s/40s creek water in non-insulated mesh trail runners risks cold feet/mild hypothermia for someone inexperienced with cold-water wading; a beginner should plan on wading boots/neoprene socks or accept wet feet only briefly and dry out fast near a fire, not as an all-day creek-panning shoe</t>
         </is>
       </c>
       <c r="Q77" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R77" s="37" t="n">
         <v>1</v>
       </c>
       <c r="S77" s="38" t="inlineStr">
         <is>
-          <t>Only use if already broken in — do not wear brand-new unbroken shoes on the trip</t>
+          <t>Only use if already broken in — do not wear brand-new unbroken shoes on the trip. Not the recommended default for beginners on this trip; pair with the neoprene wading sock / water shoe options below for cold creek work</t>
         </is>
       </c>
       <c r="T77">
@@ -19605,7 +19621,7 @@
       </c>
       <c r="I80" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/b/darn-tough/c/hiking-socks</t>
+          <t>https://www.rei.com/product/165398/rei-co-op-merino-wool-lightweight-hiking-crew-socks</t>
         </is>
       </c>
       <c r="J80" s="38" t="inlineStr">
@@ -19787,11 +19803,11 @@
         </is>
       </c>
       <c r="H82" s="40" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="I82" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/b/darn-tough/c/hiking-socks</t>
+          <t>https://www.sealskinzusa.com/products/waterproof-all-weather-mid-length-sock</t>
         </is>
       </c>
       <c r="J82" s="38" t="inlineStr">
@@ -20066,7 +20082,7 @@
       </c>
       <c r="I85" s="41" t="inlineStr">
         <is>
-          <t>https://www.treelinereview.com/gearreviews/best-lightweight-rain-jackets</t>
+          <t>https://www.rei.com/product/166198/outdoor-research-helium-rain-jacket-mens</t>
         </is>
       </c>
       <c r="J85" s="38" t="inlineStr">
@@ -20294,7 +20310,7 @@
       </c>
       <c r="S87" s="38" t="inlineStr">
         <is>
-          <t>Watch for sales — this jacket routinely drops to $115-150 | TIER ODDITY: Value ($239.00) costs more than Premium ($200.00) in this category -- kept as sourced, not auto-corrected.</t>
+          <t>Watch for sales — this jacket routinely drops to $115-150 | TIER ODDITY: Value ($239.00) costs more than Premium ($170.00) in this category -- kept as sourced, not auto-corrected.</t>
         </is>
       </c>
       <c r="T87">
@@ -20337,11 +20353,11 @@
         </is>
       </c>
       <c r="H88" s="40" t="n">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="I88" s="41" t="inlineStr">
         <is>
-          <t>https://www.adventurealan.com/enlightened-equipment-torrid-apex-jacket-review/</t>
+          <t>https://enlightenedequipment.com/mens-torrid-jacket/</t>
         </is>
       </c>
       <c r="J88" s="38" t="inlineStr">
@@ -20387,7 +20403,7 @@
       </c>
       <c r="S88" s="38" t="inlineStr">
         <is>
-          <t>Order now if going this route — cottage lead times can blow the Oct 15 deadline | TIER ODDITY: Premium ($200.00) is cheaper than Value ($239.00) in this category -- kept as sourced.</t>
+          <t>Order now if going this route — cottage lead times can blow the Oct 15 deadline | TIER ODDITY: Premium ($170.00) is cheaper than Value ($239.00) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T88">
@@ -20430,11 +20446,11 @@
         </is>
       </c>
       <c r="H89" s="40" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I89" s="41" t="inlineStr">
         <is>
-          <t>https://www.skyestoury.com/blog/fleece-mid-layers-hiking-backpacking</t>
+          <t>https://www.decathlon.com/products/mens-hiking-fleece-mh100-312361</t>
         </is>
       </c>
       <c r="J89" s="38" t="inlineStr">
@@ -20705,11 +20721,11 @@
         </is>
       </c>
       <c r="H92" s="40" t="n">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="I92" s="41" t="inlineStr">
         <is>
-          <t>https://mydroneauthority.com/best-merino-wool-base-layers/</t>
+          <t>https://merino.tech/products/men-250-base-layer-set-wool-clothing</t>
         </is>
       </c>
       <c r="J92" s="38" t="inlineStr">
@@ -20755,7 +20771,7 @@
       </c>
       <c r="S92" s="38" t="inlineStr">
         <is>
-          <t>Reserve this set exclusively as dry sleep clothes — never wear it panning</t>
+          <t>Reserve this set exclusively as dry sleep clothes — never wear it panning | TIER ODDITY: Budget ($100.00) costs more than Value ($95.00) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T92">
@@ -20846,7 +20862,11 @@
       <c r="R93" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S93" s="38" t="inlineStr"/>
+      <c r="S93" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($95.00) is cheaper than Budget ($100.00) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T93">
         <f>A93&amp;"|"&amp;C93</f>
         <v/>
@@ -20887,11 +20907,11 @@
         </is>
       </c>
       <c r="H94" s="40" t="n">
-        <v>190</v>
+        <v>235</v>
       </c>
       <c r="I94" s="41" t="inlineStr">
         <is>
-          <t>https://bettertrail.com/outdoor-gear/best-base-layers</t>
+          <t>https://www.rei.com/product/139520/icebreaker-200-oasis-half-zip-base-layer-top-mens</t>
         </is>
       </c>
       <c r="J94" s="38" t="inlineStr">
@@ -20976,11 +20996,11 @@
         </is>
       </c>
       <c r="H95" s="40" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="I95" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/learn/expert-advice/best-hiking-pants.html</t>
+          <t>https://www.rei.com/product/236137/rei-co-op-trailmade-pants-mens</t>
         </is>
       </c>
       <c r="J95" s="38" t="inlineStr">
@@ -21146,7 +21166,7 @@
       </c>
       <c r="E97" s="37" t="inlineStr">
         <is>
-          <t>Stretch Zion Cargo Pants</t>
+          <t>Stretch Zion Straight Pants (cargo version discontinued, replaced by current lineup)</t>
         </is>
       </c>
       <c r="F97" s="39" t="n">
@@ -21158,11 +21178,11 @@
         </is>
       </c>
       <c r="H97" s="40" t="n">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="I97" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/b/prana/c/mens-hiking-pants</t>
+          <t>https://www.rei.com/product/134025/prana-stretch-zion-straight-pants-mens</t>
         </is>
       </c>
       <c r="J97" s="38" t="inlineStr">
@@ -21251,7 +21271,7 @@
       </c>
       <c r="I98" s="41" t="inlineStr">
         <is>
-          <t>https://www.iheartpacificnorthwest.com/blog_post/hats-gloves-and-neck-gaiters-for-hiking/</t>
+          <t>https://www.amazon.com/Wmcaps-Winter-Beanie-Hats-for-Men-Women-Fleece-Lined-Beanie-Soft-Warm-Knit-Hat-Ski-Stocking-Cuffed-Cap/dp/B0BBZZZH84</t>
         </is>
       </c>
       <c r="J98" s="38" t="inlineStr">
@@ -21429,7 +21449,7 @@
       </c>
       <c r="I100" s="41" t="inlineStr">
         <is>
-          <t>https://www.iheartpacificnorthwest.com/blog_post/hats-gloves-and-neck-gaiters-for-hiking/</t>
+          <t>https://www.rei.com/product/217179/smartwool-merino-250-reversible-pattern-cuffed-beanie</t>
         </is>
       </c>
       <c r="J100" s="38" t="inlineStr">
@@ -21518,7 +21538,7 @@
       </c>
       <c r="I101" s="41" t="inlineStr">
         <is>
-          <t>https://www.iheartpacificnorthwest.com/blog_post/hats-gloves-and-neck-gaiters-for-hiking/</t>
+          <t>https://www.walmart.com/ip/2844295050</t>
         </is>
       </c>
       <c r="J101" s="38" t="inlineStr">
@@ -21696,7 +21716,7 @@
       </c>
       <c r="I103" s="41" t="inlineStr">
         <is>
-          <t>https://www.iheartpacificnorthwest.com/blog_post/hats-gloves-and-neck-gaiters-for-hiking/</t>
+          <t>https://opossumworld.com/collections/mens-gloves/possum-merino</t>
         </is>
       </c>
       <c r="J103" s="38" t="inlineStr">
@@ -22226,7 +22246,7 @@
       </c>
       <c r="E109" s="37" t="inlineStr">
         <is>
-          <t>Cairn Adventure Sandals</t>
+          <t>Cairn Evo Adventure Sandals (current lineup; original Cairn Adventure Sandal discontinued)</t>
         </is>
       </c>
       <c r="F109" s="39" t="n">
@@ -22242,7 +22262,7 @@
       </c>
       <c r="I109" s="41" t="inlineStr">
         <is>
-          <t>https://www.adventurealan.com/ultralight-sandals-backpacking/</t>
+          <t>https://bedrocksandals.com/products/cairn-evo</t>
         </is>
       </c>
       <c r="J109" s="38" t="inlineStr">
@@ -23055,11 +23075,11 @@
         </is>
       </c>
       <c r="H118" s="40" t="n">
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="I118" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/learn/expert-advice/best-hiking-pants.html</t>
+          <t>https://fishwest.com/products/simms-tributary-stockingfoot-waders-mens</t>
         </is>
       </c>
       <c r="J118" s="38" t="inlineStr">
@@ -23245,7 +23265,7 @@
       </c>
       <c r="I120" s="41" t="inlineStr">
         <is>
-          <t>https://www.goldprospectors.org/Forum/aft/9275</t>
+          <t>https://www.amazon.com/NoCry-Home-Gardening-Knee-Pads/dp/B06XJ2BFW7</t>
         </is>
       </c>
       <c r="J120" s="38" t="inlineStr">
@@ -23837,11 +23857,11 @@
         <v>4</v>
       </c>
       <c r="R126" s="37" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="S126" s="38" t="inlineStr">
         <is>
-          <t>Could be one shared set at the base-camp pan-out station rather than one per person</t>
+          <t>One shared set at the base-camp pan-out station, split 6 ways, rather than one per person</t>
         </is>
       </c>
       <c r="T126">
@@ -24786,11 +24806,11 @@
         </is>
       </c>
       <c r="H137" s="40" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="I137" s="41" t="inlineStr">
         <is>
-          <t>https://ukgoldprospector.co.uk/news/best-equipment-gold-prospecting-uk.html</t>
+          <t>https://www.amazon.com/Magnifier-Portable-Keychain-Diamonds-Antiques/dp/B09B1ZBY47</t>
         </is>
       </c>
       <c r="J137" s="38" t="inlineStr">
@@ -24834,7 +24854,11 @@
       <c r="R137" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S137" s="38" t="inlineStr"/>
+      <c r="S137" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Budget ($19.00) costs more than Value ($13.00) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T137">
         <f>A137&amp;"|"&amp;C137</f>
         <v/>
@@ -24923,7 +24947,11 @@
       <c r="R138" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S138" s="38" t="inlineStr"/>
+      <c r="S138" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($13.00) is cheaper than Budget ($19.00) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T138">
         <f>A138&amp;"|"&amp;C138</f>
         <v/>
@@ -24964,11 +24992,11 @@
         </is>
       </c>
       <c r="H139" s="40" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="I139" s="41" t="inlineStr">
         <is>
-          <t>https://ukgoldprospector.co.uk/news/best-equipment-gold-prospecting-uk.html</t>
+          <t>https://cooltools.us/products/loupe-triplet-10x</t>
         </is>
       </c>
       <c r="J139" s="38" t="inlineStr">
@@ -25053,11 +25081,11 @@
         </is>
       </c>
       <c r="H140" s="40" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I140" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/613426092</t>
+          <t>https://www.walmart.com/ip/Fiskars-Indoor-and-More-Garden-Trowel-Soil-Scoop-Black/5371466767</t>
         </is>
       </c>
       <c r="J140" s="38" t="inlineStr">
@@ -25146,7 +25174,7 @@
         </is>
       </c>
       <c r="H141" s="40" t="n">
-        <v>22.5</v>
+        <v>20.95</v>
       </c>
       <c r="I141" s="41" t="inlineStr">
         <is>
@@ -25851,7 +25879,7 @@
       </c>
       <c r="B149" s="38" t="inlineStr">
         <is>
-          <t>30F-rated sleeping bag/quilt (RECOMMENDED default)</t>
+          <t>30F-rated sleeping bag/quilt (RECOMMENDED default -- beginner-safe pick)</t>
         </is>
       </c>
       <c r="C149" s="37" t="inlineStr">
@@ -25928,7 +25956,7 @@
       </c>
       <c r="S149" s="38" t="inlineStr">
         <is>
-          <t>NEW group added 2026-09-21 alongside the existing 20F group per updated weather research; recommended DEFAULT pick for this trip</t>
+          <t>NEW group added 2026-09-21 alongside the existing 20F group per updated weather research; RECOMMENDED DEFAULT pick for this trip -- zippered synthetic bag is the beginner-safe choice for freezing/damp deer-season nights (no draft-sealing technique to learn)</t>
         </is>
       </c>
       <c r="T149">
@@ -25944,7 +25972,7 @@
       </c>
       <c r="B150" s="38" t="inlineStr">
         <is>
-          <t>30F-rated sleeping bag/quilt (RECOMMENDED default)</t>
+          <t>30F-rated sleeping bag/quilt (upgrade option, not the default -- BEGINNER CAUTION: quilt)</t>
         </is>
       </c>
       <c r="C150" s="37" t="inlineStr">
@@ -26021,7 +26049,7 @@
       </c>
       <c r="S150" s="38" t="inlineStr">
         <is>
-          <t>NEW group added 2026-09-21; recommended DEFAULT pick — best weight/cost balance for this trip's actual verified temps</t>
+          <t>NEW group added 2026-09-21; BEGINNER CAUTION -- quilts have no zipper/hood and rely on a correct pad seal to avoid drafts; risky for a first cold-weather trip if unpracticed. Best weight/cost balance IF the group is comfortable with a quilt, but the Budget synthetic bag above is the safer default for beginners.</t>
         </is>
       </c>
       <c r="T150">
@@ -26037,7 +26065,7 @@
       </c>
       <c r="B151" s="38" t="inlineStr">
         <is>
-          <t>30F-rated sleeping bag/quilt (RECOMMENDED default)</t>
+          <t>30F-rated sleeping bag/quilt (upgrade option, not the default -- BEGINNER CAUTION: quilt)</t>
         </is>
       </c>
       <c r="C151" s="37" t="inlineStr">

</xml_diff>

<commit_message>
Fix verified link-check price mismatches (gold pan, beanie, crevice tool set)
Spot-checked ~90+ BUY_LIST.md product links via WebFetch/browser. Corrected
three confirmed price mismatches (>15%) in gear-tiers-clothing-panning.json:
Garrett gold pan $16->$8.99, FarPointe Alpha Drifter beanie $28->$38, and the
value-tier crevice tool set $16->$59.95 (link actually goes to a $59.95
kit, not $16). Rebuilt BUY_LIST.md/Gear_Picker.xlsx/index.html.

Several other links were found broken/stale during the check (dead Amazon
ASINs, out-of-stock direct-brand pages, an ASR classifier blog link instead
of a product page, an expired Slickdeals coupon link) but were not fixed in
this pass due to time constraints -- flagged for follow-up.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gear_Picker.xlsx
+++ b/Gear_Picker.xlsx
@@ -9996,7 +9996,7 @@
         <v>0.7</v>
       </c>
       <c r="N35" s="34" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="O35" s="11" t="inlineStr">
         <is>
@@ -11028,7 +11028,7 @@
         <v>10</v>
       </c>
       <c r="N43" s="34" t="n">
-        <v>16</v>
+        <v>8.99</v>
       </c>
       <c r="O43" s="11" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         <v>6</v>
       </c>
       <c r="N46" s="34" t="n">
-        <v>16</v>
+        <v>59.95</v>
       </c>
       <c r="O46" s="11" t="inlineStr">
         <is>
@@ -21363,7 +21363,7 @@
         </is>
       </c>
       <c r="H99" s="40" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="I99" s="41" t="inlineStr">
         <is>
@@ -21411,7 +21411,11 @@
       <c r="R99" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S99" s="38" t="inlineStr"/>
+      <c r="S99" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($38.00) costs more than Premium ($35.00) in this category -- kept as sourced, not auto-corrected.</t>
+        </is>
+      </c>
       <c r="T99">
         <f>A99&amp;"|"&amp;C99</f>
         <v/>
@@ -21500,7 +21504,11 @@
       <c r="R100" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S100" s="38" t="inlineStr"/>
+      <c r="S100" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Premium ($35.00) is cheaper than Value ($38.00) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T100">
         <f>A100&amp;"|"&amp;C100</f>
         <v/>
@@ -23496,7 +23504,7 @@
       </c>
       <c r="S122" s="38" t="inlineStr">
         <is>
-          <t>Great for beginners; experienced members of the group may prefer the value-tier Garrett</t>
+          <t>Great for beginners; experienced members of the group may prefer the value-tier Garrett | TIER ODDITY: Budget ($9.00) costs more than Value ($8.99) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T122">
@@ -23539,7 +23547,7 @@
         </is>
       </c>
       <c r="H123" s="40" t="n">
-        <v>16</v>
+        <v>8.99</v>
       </c>
       <c r="I123" s="41" t="inlineStr">
         <is>
@@ -23589,7 +23597,7 @@
       </c>
       <c r="S123" s="38" t="inlineStr">
         <is>
-          <t>This is the pan genuinely worth buying one of per person if budget allows even a small step up from bare-minimum</t>
+          <t>This is the pan genuinely worth buying one of per person if budget allows even a small step up from bare-minimum | TIER ODDITY: Value ($8.99) is cheaper than Budget ($9.00) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T123">
@@ -24360,7 +24368,7 @@
         </is>
       </c>
       <c r="H132" s="40" t="n">
-        <v>16</v>
+        <v>59.95</v>
       </c>
       <c r="I132" s="41" t="inlineStr">
         <is>
@@ -24408,7 +24416,11 @@
       <c r="R132" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S132" s="38" t="inlineStr"/>
+      <c r="S132" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Value ($59.95) costs more than Premium ($25.00) in this category -- kept as sourced, not auto-corrected.</t>
+        </is>
+      </c>
       <c r="T132">
         <f>A132&amp;"|"&amp;C132</f>
         <v/>
@@ -24497,7 +24509,11 @@
       <c r="R133" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S133" s="38" t="inlineStr"/>
+      <c r="S133" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Premium ($25.00) is cheaper than Value ($59.95) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T133">
         <f>A133&amp;"|"&amp;C133</f>
         <v/>

</xml_diff>

<commit_message>
Replace 9 more dead/wrong-product links (kitchen-water-elec, clothing-panning, extras-food), merge pending price-check CSVs, rebuild picker/buy list/hub
- kitchen-water-elec.json: Sea to Summit spoon, Katadyn BeFree (now AC variant, +$8), Equate toiletry kit (cheaper replacement), Cascade Mountain Tech poles (+$13), Therm-a-Rest Z Seat (renamed, +$14.33)
- Merged 3 pending price-check CSVs (149 rows) into price-check-2026-09.csv, applied 17 verified price changes + 5 sleep-temp dead-link fixes from a prior session
- Re-ran build_gear_picker.py -> build_buy_list.py -> build_hub.py so Gear_Picker.xlsx, BUY_LIST.md, and index.html's Buy tab all reflect the corrected prices/links (SOLID total/person $2,329.83 -> $2,473.52)
- Ignore tools/__pycache__/
</commit_message>
<xml_diff>
--- a/Gear_Picker.xlsx
+++ b/Gear_Picker.xlsx
@@ -7496,7 +7496,7 @@
         <v>2.3</v>
       </c>
       <c r="N15" s="34" t="n">
-        <v>44.95</v>
+        <v>52.95</v>
       </c>
       <c r="O15" s="11" t="inlineStr">
         <is>
@@ -7586,7 +7586,7 @@
         <v>1.6</v>
       </c>
       <c r="E16" s="34" t="n">
-        <v>2</v>
+        <v>2.17</v>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
@@ -8618,7 +8618,7 @@
         <v>1.5</v>
       </c>
       <c r="E24" s="34" t="n">
-        <v>4.25</v>
+        <v>8.75</v>
       </c>
       <c r="F24" s="11" t="inlineStr">
         <is>
@@ -8747,7 +8747,7 @@
         <v>3.5</v>
       </c>
       <c r="E25" s="34" t="n">
-        <v>6</v>
+        <v>3.94</v>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
@@ -8876,7 +8876,7 @@
         <v>18</v>
       </c>
       <c r="E26" s="34" t="n">
-        <v>39.99</v>
+        <v>49.99</v>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
@@ -8915,7 +8915,7 @@
         <v>8.1</v>
       </c>
       <c r="N26" s="34" t="n">
-        <v>51.98</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="O26" s="11" t="inlineStr">
         <is>
@@ -9044,7 +9044,7 @@
         <v>2</v>
       </c>
       <c r="N27" s="34" t="n">
-        <v>19.95</v>
+        <v>34.28</v>
       </c>
       <c r="O27" s="11" t="inlineStr">
         <is>
@@ -9392,7 +9392,7 @@
         <v>2.5</v>
       </c>
       <c r="E30" s="34" t="n">
-        <v>18</v>
+        <v>8.83</v>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
@@ -9560,7 +9560,7 @@
         <v>12.5</v>
       </c>
       <c r="N31" s="34" t="n">
-        <v>100</v>
+        <v>99.95</v>
       </c>
       <c r="O31" s="11" t="inlineStr">
         <is>
@@ -9689,7 +9689,7 @@
         <v>11.6</v>
       </c>
       <c r="N32" s="34" t="n">
-        <v>239</v>
+        <v>118.99</v>
       </c>
       <c r="O32" s="11" t="inlineStr">
         <is>
@@ -9947,7 +9947,7 @@
         <v>10</v>
       </c>
       <c r="N34" s="34" t="n">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="O34" s="11" t="inlineStr">
         <is>
@@ -10166,7 +10166,7 @@
         <v>2</v>
       </c>
       <c r="E36" s="34" t="n">
-        <v>10</v>
+        <v>14.99</v>
       </c>
       <c r="F36" s="11" t="inlineStr">
         <is>
@@ -10334,7 +10334,7 @@
         <v>2.3</v>
       </c>
       <c r="N37" s="34" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="O37" s="11" t="inlineStr">
         <is>
@@ -10682,7 +10682,7 @@
         <v>6</v>
       </c>
       <c r="E40" s="34" t="n">
-        <v>10</v>
+        <v>17.37</v>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
@@ -10721,7 +10721,7 @@
         <v>7</v>
       </c>
       <c r="N40" s="34" t="n">
-        <v>18</v>
+        <v>14.99</v>
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
@@ -11069,7 +11069,7 @@
         <v>5</v>
       </c>
       <c r="E43" s="34" t="n">
-        <v>8</v>
+        <v>8.99</v>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
@@ -11495,7 +11495,7 @@
         <v>2</v>
       </c>
       <c r="N46" s="34" t="n">
-        <v>9</v>
+        <v>11.99</v>
       </c>
       <c r="O46" s="11" t="inlineStr">
         <is>
@@ -11843,7 +11843,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="34" t="n">
-        <v>19</v>
+        <v>7.99</v>
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
@@ -11882,7 +11882,7 @@
         <v>2.5</v>
       </c>
       <c r="N49" s="34" t="n">
-        <v>13</v>
+        <v>8.98</v>
       </c>
       <c r="O49" s="11" t="inlineStr">
         <is>
@@ -11972,7 +11972,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="34" t="n">
-        <v>9</v>
+        <v>6.28</v>
       </c>
       <c r="F50" s="11" t="inlineStr">
         <is>
@@ -12230,7 +12230,7 @@
         <v>30</v>
       </c>
       <c r="E52" s="34" t="n">
-        <v>45</v>
+        <v>7.26</v>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
@@ -12308,7 +12308,7 @@
         <v>52</v>
       </c>
       <c r="W52" s="34" t="n">
-        <v>95</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="X52" s="11" t="inlineStr">
         <is>
@@ -15809,7 +15809,7 @@
       </c>
       <c r="I36" s="41" t="inlineStr">
         <is>
-          <t>https://seatosummit.com/products/alpha-light-utensil-long-spoon</t>
+          <t>https://www.amazon.com/dp/B0CWVSLQ4J</t>
         </is>
       </c>
       <c r="J36" s="38" t="inlineStr">
@@ -15855,7 +15855,7 @@
       </c>
       <c r="S36" s="38" t="inlineStr">
         <is>
-          <t>TIER ODDITY: Value ($10.95) costs more than Premium ($9.95) in this category -- kept as sourced, not auto-corrected.</t>
+          <t>seatosummit.com product page is dead (site sells nothing directly); replacement is the same Frontier Ultralight Long Handle Spoon on Amazon, same $10.95 price. | TIER ODDITY: Value ($10.95) costs more than Premium ($9.95) in this category -- kept as sourced, not auto-corrected.</t>
         </is>
       </c>
       <c r="T36">
@@ -16041,7 +16041,7 @@
       </c>
       <c r="S38" s="38" t="inlineStr">
         <is>
-          <t>Group share $5.00 | SAFETY NOTE (added 2026-09-23): sleep with it below freezing -- a wetted Sawyer membrane cracks if it freezes, so it must go inside the sleeping bag with you on any night near/below 32F, not left in a pack pocket. Cheap chemical backup already on the buy list: Aquatabs 30-pack (research/gear-tiers-extras-food.json, section A -- water_treatment_backup, https://www.rei.com/product/109906/aquatabs-water-purification-tablets-package-of-30) covers the group if the filter ever fails. | TIER ODDITY: Budget ($45.95) costs more than Value ($44.95) in this category -- kept as sourced.</t>
+          <t>Group share $5.00 | SAFETY NOTE (added 2026-09-23): sleep with it below freezing -- a wetted Sawyer membrane cracks if it freezes, so it must go inside the sleeping bag with you on any night near/below 32F, not left in a pack pocket. Cheap chemical backup already on the buy list: Aquatabs 30-pack (research/gear-tiers-extras-food.json, section A -- water_treatment_backup, https://www.rei.com/product/109906/aquatabs-water-purification-tablets-package-of-30) covers the group if the filter ever fails.</t>
         </is>
       </c>
       <c r="T38">
@@ -16084,11 +16084,11 @@
         </is>
       </c>
       <c r="H39" s="40" t="n">
-        <v>44.95</v>
+        <v>52.95</v>
       </c>
       <c r="I39" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/116364/katadyn-befree-10-l-water-filter-bottle-338-fl-oz</t>
+          <t>https://www.rei.com/product/247273/katadyn-befree-ac-10-l-water-filter-bottle</t>
         </is>
       </c>
       <c r="J39" s="38" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="S39" s="38" t="inlineStr">
         <is>
-          <t>Group share $7.49 | SAFETY NOTE (added 2026-09-23): sleep with it below freezing -- same hollow-fiber freeze-crack risk as the Sawyer, keep it in the sleeping bag on any night near/below 32F. Cheap chemical backup already on the buy list: Aquatabs 30-pack (research/gear-tiers-extras-food.json, section A, https://www.rei.com/product/109906/aquatabs-water-purification-tablets-package-of-30). | TIER ODDITY: Value ($44.95) is cheaper than Budget ($45.95) in this category -- kept as sourced.</t>
+          <t>Group share $8.83 | SAFETY NOTE (added 2026-09-23): sleep with it below freezing -- same hollow-fiber freeze-crack risk as the Sawyer, keep it in the sleeping bag on any night near/below 32F. Cheap chemical backup already on the buy list: Aquatabs 30-pack (research/gear-tiers-extras-food.json, section A, https://www.rei.com/product/109906/aquatabs-water-purification-tablets-package-of-30). Old plain BeFree 1.0L listing (product 116364) is dead; REI now only sells the BeFree AC version (adds activated carbon for taste/odor), $52.95 not $44.95 -- price jump is real, not a mispick.</t>
         </is>
       </c>
       <c r="T39">
@@ -16270,7 +16270,7 @@
         </is>
       </c>
       <c r="H41" s="40" t="n">
-        <v>2</v>
+        <v>2.17</v>
       </c>
       <c r="I41" s="41" t="inlineStr">
         <is>
@@ -18474,7 +18474,7 @@
         </is>
       </c>
       <c r="H65" s="40" t="n">
-        <v>4.25</v>
+        <v>8.75</v>
       </c>
       <c r="I65" s="41" t="inlineStr">
         <is>
@@ -18524,7 +18524,7 @@
       </c>
       <c r="S65" s="38" t="inlineStr">
         <is>
-          <t>Split 6 ways (shared cathole trowel, carried on the overnight leg)</t>
+          <t>Split 6 ways (shared cathole trowel, carried on the overnight leg) | TIER ODDITY: Budget ($8.75) costs more than Value ($7.95) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T65">
@@ -18617,7 +18617,7 @@
       </c>
       <c r="S66" s="38" t="inlineStr">
         <is>
-          <t>Split 6 ways (shared cathole trowel, carried on the overnight leg)</t>
+          <t>Split 6 ways (shared cathole trowel, carried on the overnight leg) | TIER ODDITY: Value ($7.95) is cheaper than Budget ($8.75) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T66">
@@ -18753,11 +18753,11 @@
         </is>
       </c>
       <c r="H68" s="40" t="n">
-        <v>6</v>
+        <v>3.94</v>
       </c>
       <c r="I68" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/Equate-Travel-Size-Toiletry-Kit/</t>
+          <t>https://www.walmart.com/ip/Equate-Travel-Kit-8-Piece-Plastics/831029303</t>
         </is>
       </c>
       <c r="J68" s="38" t="inlineStr">
@@ -18799,7 +18799,7 @@
       </c>
       <c r="S68" s="38" t="inlineStr">
         <is>
-          <t>Personal, full price -- each hiker buys/packs their own</t>
+          <t>Personal, full price -- each hiker buys/packs their own. Old direct-slug URL didn't resolve; replacement is Equate's current 8-Piece Travel Kit (empty refillable bottles, not toothbrush/toothpaste/TP bundled) at its real product ID, $3.94 not $6.00 -- fill it with the toothbrush kit and TP already on the buy list.</t>
         </is>
       </c>
       <c r="T68">
@@ -19020,7 +19020,7 @@
         </is>
       </c>
       <c r="H71" s="40" t="n">
-        <v>39.99</v>
+        <v>49.99</v>
       </c>
       <c r="I71" s="41" t="inlineStr">
         <is>
@@ -19109,11 +19109,11 @@
         </is>
       </c>
       <c r="H72" s="40" t="n">
-        <v>51.98</v>
+        <v>64.98999999999999</v>
       </c>
       <c r="I72" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Cascade-Mountain-Tech-Carbon-Trekking/dp/B07RH3P6MT</t>
+          <t>https://www.amazon.com/dp/B07S4DRDNT</t>
         </is>
       </c>
       <c r="J72" s="38" t="inlineStr">
@@ -19157,7 +19157,11 @@
       <c r="R72" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S72" s="38" t="inlineStr"/>
+      <c r="S72" s="38" t="inlineStr">
+        <is>
+          <t>Old ASIN listing is dead; replacement is the current Cascade Mountain Tech Carbon Fiber Quick Lock poles listing, same product line, $64.99 not $51.98 -- flagging the jump.</t>
+        </is>
+      </c>
       <c r="T72">
         <f>A72&amp;"|"&amp;C72</f>
         <v/>
@@ -19376,11 +19380,11 @@
         </is>
       </c>
       <c r="H75" s="40" t="n">
-        <v>19.95</v>
+        <v>34.28</v>
       </c>
       <c r="I75" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/734520/therm-a-rest-z-seat</t>
+          <t>https://www.amazon.com/dp/B07MV959N6</t>
         </is>
       </c>
       <c r="J75" s="38" t="inlineStr">
@@ -19424,7 +19428,11 @@
       <c r="R75" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S75" s="38" t="inlineStr"/>
+      <c r="S75" s="38" t="inlineStr">
+        <is>
+          <t>Old REI product ID dead; renamed "Z Seat Cushion Insulated Sitting Pad" -- replacement is the same product on Amazon (REI access-blocked on repeated checks), $34.28 not $19.95 -- flagging the jump. | TIER ODDITY: Value ($34.28) costs more than Premium ($22.50) in this category -- kept as sourced, not auto-corrected.</t>
+        </is>
+      </c>
       <c r="T75">
         <f>A75&amp;"|"&amp;C75</f>
         <v/>
@@ -19513,7 +19521,11 @@
       <c r="R76" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S76" s="38" t="inlineStr"/>
+      <c r="S76" s="38" t="inlineStr">
+        <is>
+          <t>TIER ODDITY: Premium ($22.50) is cheaper than Value ($34.28) in this category -- kept as sourced.</t>
+        </is>
+      </c>
       <c r="T76">
         <f>A76&amp;"|"&amp;C76</f>
         <v/>
@@ -20104,7 +20116,7 @@
         </is>
       </c>
       <c r="H83" s="40" t="n">
-        <v>18</v>
+        <v>8.83</v>
       </c>
       <c r="I83" s="41" t="inlineStr">
         <is>
@@ -20476,11 +20488,11 @@
         </is>
       </c>
       <c r="H87" s="40" t="n">
-        <v>100</v>
+        <v>99.95</v>
       </c>
       <c r="I87" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/127336/rei-co-op-rainier-rain-jacket-mens</t>
+          <t>https://www.rei.com/product/227570/rei-co-op-rainier-rain-jacket-mens</t>
         </is>
       </c>
       <c r="J87" s="38" t="inlineStr">
@@ -20524,7 +20536,11 @@
       <c r="R87" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S87" s="38" t="inlineStr"/>
+      <c r="S87" s="38" t="inlineStr">
+        <is>
+          <t>Old listing (#127336) is discontinued; replacement is the current-generation Rainier Rain Jacket (#227570), same name/role/price point (product #127336 no longer sold).</t>
+        </is>
+      </c>
       <c r="T87">
         <f>A87&amp;"|"&amp;C87</f>
         <v/>
@@ -20747,7 +20763,7 @@
         </is>
       </c>
       <c r="H90" s="40" t="n">
-        <v>239</v>
+        <v>118.99</v>
       </c>
       <c r="I90" s="41" t="inlineStr">
         <is>
@@ -20797,7 +20813,7 @@
       </c>
       <c r="S90" s="38" t="inlineStr">
         <is>
-          <t>Watch for sales — this jacket routinely drops to $115-150 | TIER ODDITY: Value ($239.00) costs more than Premium ($170.00) in this category -- kept as sourced, not auto-corrected.</t>
+          <t>Watch for sales — this jacket routinely drops to $115-150</t>
         </is>
       </c>
       <c r="T90">
@@ -20890,7 +20906,7 @@
       </c>
       <c r="S91" s="38" t="inlineStr">
         <is>
-          <t>Order now if going this route — cottage lead times can blow the Oct 15 deadline | TIER ODDITY: Premium ($170.00) is cheaper than Value ($239.00) in this category -- kept as sourced.</t>
+          <t>Order now if going this route — cottage lead times can blow the Oct 15 deadline</t>
         </is>
       </c>
       <c r="T91">
@@ -21258,7 +21274,7 @@
       </c>
       <c r="S95" s="38" t="inlineStr">
         <is>
-          <t>Reserve this set exclusively as dry sleep clothes — never wear it panning | TIER ODDITY: Budget ($100.00) costs more than Value ($95.00) in this category -- kept as sourced.</t>
+          <t>Reserve this set exclusively as dry sleep clothes — never wear it panning</t>
         </is>
       </c>
       <c r="T95">
@@ -21301,7 +21317,7 @@
         </is>
       </c>
       <c r="H96" s="40" t="n">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="I96" s="41" t="inlineStr">
         <is>
@@ -21349,11 +21365,7 @@
       <c r="R96" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S96" s="38" t="inlineStr">
-        <is>
-          <t>TIER ODDITY: Value ($95.00) is cheaper than Budget ($100.00) in this category -- kept as sourced.</t>
-        </is>
-      </c>
+      <c r="S96" s="38" t="inlineStr"/>
       <c r="T96">
         <f>A96&amp;"|"&amp;C96</f>
         <v/>
@@ -21762,7 +21774,7 @@
         </is>
       </c>
       <c r="H101" s="40" t="n">
-        <v>10</v>
+        <v>14.99</v>
       </c>
       <c r="I101" s="41" t="inlineStr">
         <is>
@@ -22126,11 +22138,11 @@
         </is>
       </c>
       <c r="H105" s="40" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="I105" s="41" t="inlineStr">
         <is>
-          <t>https://www.rei.com/product/871650/outdoor-research-pl-400-sensor-gloves-mens</t>
+          <t>https://www.rei.com/product/C08576/outdoor-research-trail-mix-xt-gloves-mens</t>
         </is>
       </c>
       <c r="J105" s="38" t="inlineStr">
@@ -22174,7 +22186,11 @@
       <c r="R105" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="S105" s="38" t="inlineStr"/>
+      <c r="S105" s="38" t="inlineStr">
+        <is>
+          <t>Replacement is Outdoor Research Trail Mix XT Gloves, recycled fleece liner glove, not the PL 400 Sensor Gloves (PL 400 no longer sold).</t>
+        </is>
+      </c>
       <c r="T105">
         <f>A105&amp;"|"&amp;C105</f>
         <v/>
@@ -22850,11 +22866,11 @@
         </is>
       </c>
       <c r="H113" s="40" t="n">
-        <v>10</v>
+        <v>17.37</v>
       </c>
       <c r="I113" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/SHOWA-Showa-620L-09-1-Pair/dp/B000VNO2BE</t>
+          <t>https://www.amazon.com/620-Coated-Liquid-Chemical-Resistant/dp/B002PJ0WRK</t>
         </is>
       </c>
       <c r="J113" s="38" t="inlineStr">
@@ -22900,7 +22916,7 @@
       </c>
       <c r="S113" s="38" t="inlineStr">
         <is>
-          <t>Order true to hand size; too small and they crack, too large and dexterity for panning suffers</t>
+          <t>Order true to hand size; too small and they crack, too large and dexterity for panning suffers. Replacement listing is the same Atlas 620 model, Small/Orange, from a different seller (original ASIN listing no longer has a valid buyable price). | TIER ODDITY: Budget ($17.37) costs more than Value ($14.99) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T113">
@@ -22943,7 +22959,7 @@
         </is>
       </c>
       <c r="H114" s="40" t="n">
-        <v>18</v>
+        <v>14.99</v>
       </c>
       <c r="I114" s="41" t="inlineStr">
         <is>
@@ -22993,7 +23009,7 @@
       </c>
       <c r="S114" s="38" t="inlineStr">
         <is>
-          <t>Pair with a thin liner glove for the coldest mornings</t>
+          <t>Pair with a thin liner glove for the coldest mornings | TIER ODDITY: Value ($14.99) is cheaper than Budget ($17.37) in this category -- kept as sourced.</t>
         </is>
       </c>
       <c r="T114">
@@ -23679,7 +23695,7 @@
         </is>
       </c>
       <c r="H122" s="40" t="n">
-        <v>8</v>
+        <v>8.99</v>
       </c>
       <c r="I122" s="41" t="inlineStr">
         <is>
@@ -24601,11 +24617,11 @@
         </is>
       </c>
       <c r="H132" s="40" t="n">
-        <v>9</v>
+        <v>11.99</v>
       </c>
       <c r="I132" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Panning-Sniffer-Snuffer-Bottle-Tweezer/dp/B0D38QYGYR</t>
+          <t>https://www.amazon.com/Mining-Clean-Snuffer-Suction-Tweezers/dp/B01NBXHLVA</t>
         </is>
       </c>
       <c r="J132" s="38" t="inlineStr">
@@ -24649,7 +24665,11 @@
       <c r="R132" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="S132" s="38" t="inlineStr"/>
+      <c r="S132" s="38" t="inlineStr">
+        <is>
+          <t>Replacement is APGOLF's single Clean Up Kit (vials + snuffer + tweezers), not a 2-pack glass-tip snuffer (the 2-pack glass-tip bottle w/ tweezers is no longer sold by any live Amazon listing).</t>
+        </is>
+      </c>
       <c r="T132">
         <f>A132&amp;"|"&amp;C132</f>
         <v/>
@@ -25329,11 +25349,11 @@
         </is>
       </c>
       <c r="H140" s="40" t="n">
-        <v>19</v>
+        <v>7.99</v>
       </c>
       <c r="I140" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Magnifier-Portable-Keychain-Diamonds-Antiques/dp/B09B1ZBY47</t>
+          <t>https://www.amazon.com/Keychain-Magnifier-Portable-Foldable-Magnifying/dp/B07RVF35W4</t>
         </is>
       </c>
       <c r="J140" s="38" t="inlineStr">
@@ -25379,7 +25399,7 @@
       </c>
       <c r="S140" s="38" t="inlineStr">
         <is>
-          <t>TIER ODDITY: Budget ($19.00) costs more than Value ($13.00) in this category -- kept as sourced.</t>
+          <t>Replacement is Rongon 10x metal folding keychain loupe, not the original plastic keychain magnifier (original listing no longer sold).</t>
         </is>
       </c>
       <c r="T140">
@@ -25422,7 +25442,7 @@
         </is>
       </c>
       <c r="H141" s="40" t="n">
-        <v>13</v>
+        <v>8.98</v>
       </c>
       <c r="I141" s="41" t="inlineStr">
         <is>
@@ -25470,11 +25490,7 @@
       <c r="R141" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="S141" s="38" t="inlineStr">
-        <is>
-          <t>TIER ODDITY: Value ($13.00) is cheaper than Budget ($19.00) in this category -- kept as sourced.</t>
-        </is>
-      </c>
+      <c r="S141" s="38" t="inlineStr"/>
       <c r="T141">
         <f>A141&amp;"|"&amp;C141</f>
         <v/>
@@ -25604,7 +25620,7 @@
         </is>
       </c>
       <c r="H143" s="40" t="n">
-        <v>9</v>
+        <v>6.28</v>
       </c>
       <c r="I143" s="41" t="inlineStr">
         <is>
@@ -26150,7 +26166,7 @@
         </is>
       </c>
       <c r="H149" s="40" t="n">
-        <v>45</v>
+        <v>7.26</v>
       </c>
       <c r="I149" s="41" t="inlineStr">
         <is>
@@ -26200,7 +26216,7 @@
       </c>
       <c r="S149" s="38" t="inlineStr">
         <is>
-          <t>Pack in a mesh bag separate from dry gear per the two-bag wet/dry system in Section C of the main gear plan | TIER ODDITY: Budget ($45.00) costs more than Value ($40.00) in this category -- kept as sourced.</t>
+          <t>Pack in a mesh bag separate from dry gear per the two-bag wet/dry system in Section C of the main gear plan</t>
         </is>
       </c>
       <c r="T149">
@@ -26293,7 +26309,7 @@
       </c>
       <c r="S150" s="38" t="inlineStr">
         <is>
-          <t>Confirm before buying that the kit's non-sluice parts alone meet your needs — don't pay for parts you can't legally use here | TIER ODDITY: Value ($40.00) is cheaper than Budget ($45.00) in this category -- kept as sourced.</t>
+          <t>Confirm before buying that the kit's non-sluice parts alone meet your needs — don't pay for parts you can't legally use here</t>
         </is>
       </c>
       <c r="T150">
@@ -26336,11 +26352,11 @@
         </is>
       </c>
       <c r="H151" s="40" t="n">
-        <v>95</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="I151" s="41" t="inlineStr">
         <is>
-          <t>https://garrett.com/garrett-14-gold-trap-pan/</t>
+          <t>https://www.amazon.com/Garrett-Deluxe-Gold-Pan-Kit/dp/B01LZI4OWD</t>
         </is>
       </c>
       <c r="J151" s="38" t="inlineStr">
@@ -26386,7 +26402,7 @@
       </c>
       <c r="S151" s="38" t="inlineStr">
         <is>
-          <t>Assemble this from the individual premium/value picks above rather than buying a single bundled product</t>
+          <t>Assemble this from the individual premium/value picks above rather than buying a single bundled product. Old garrett.com link now resolves to just the bare 14" pan ($8.99), not a bundle -- replacement is the real Garrett Deluxe Gold Pan Kit (9-piece: 4 pans, classifier, snuffer bottle, tweezers, magnifier) sold on Amazon, the closest verified in-stock equivalent to this curated bundle (no exact stainless-crevice-tools + mesh-sack combo is currently sold as a single product).</t>
         </is>
       </c>
       <c r="T151">

</xml_diff>

<commit_message>
Set Captain's picks for gloves/knee-pads/waders, rebuild buy list
Glacier Glove Kenai Original neoprene gloves ($24.99, dexterity over
staying dry), Bodyprox strap-on knee pads ($15.99, Captain's own find),
Frogg Toggs Canyon II breathable hip waders ($98.29, upgrade from the
rubber/PVC Hodgman pick). Live prices verified in-browser. Rebuilt via
build_gear_picker.py -> build_buy_list.py -> build_hub.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Gear_Picker.xlsx
+++ b/Gear_Picker.xlsx
@@ -10675,14 +10675,14 @@
       </c>
       <c r="C40" s="32" t="inlineStr">
         <is>
-          <t>Atlas 620 PVC-Coated Gauntlet Glove</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E40" s="34" t="n">
-        <v>17.37</v>
+        <v>24.99</v>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>TreasureNet and prospecting forums repeatedly recommend cheap PVC-dipped work gloves like the Atlas 620 for cold-water panning — a fleece-lined double-dipped PVC glove originally designed for the Alaskan fishing trade, giving real cold/wet protection for around $10.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
@@ -10714,14 +10714,14 @@
       </c>
       <c r="L40" s="35" t="inlineStr">
         <is>
-          <t>24" Rubber Gauntlet Gloves, Texturized Palm</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="M40" s="33" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N40" s="34" t="n">
-        <v>14.99</v>
+        <v>24.99</v>
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
@@ -10738,7 +10738,7 @@
       </c>
       <c r="R40" s="11" t="inlineStr">
         <is>
-          <t>Purpose-marketed for gold panning specifically, with a longer 24" gauntlet that leaves interior room for a thin knit or fleece glove liner underneath for extra warmth in cold conditions — a step up from generic work gloves at a similar price.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="S40" s="11" t="inlineStr">
@@ -10972,18 +10972,18 @@
       </c>
       <c r="L42" s="35" t="inlineStr">
         <is>
-          <t>Mackenzie Cleated Hip Bootfoot Fishing Wader</t>
+          <t>Canyon II Stockingfoot Hip Wader, Medium (needs separate wading shoe)</t>
         </is>
       </c>
       <c r="M42" s="33" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="N42" s="34" t="n">
-        <v>43.51</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="O42" s="11" t="inlineStr">
         <is>
-          <t>$20-30 used</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="P42" s="11" t="n">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="R42" s="11" t="inlineStr">
         <is>
-          <t>Hip waders show up in wading/fishing gear guides as an affordable step up for anyone who wants to stand in deeper pools without soaking pants — useful if scouting deeper holes, though most panning happens in water too shallow to need them.</t>
+          <t>Breathable upgrade over the rubber/PVC Hodgman pick -- highest-rated breathable hip wader at this size, and hip height already exceeds what shin-deep hand-panning needs. Needs a separate wading shoe (not bundled).</t>
         </is>
       </c>
       <c r="S42" s="11" t="inlineStr">
@@ -11062,18 +11062,18 @@
       </c>
       <c r="C43" s="32" t="inlineStr">
         <is>
-          <t>Foam Gardening Knee Pad</t>
+          <t>Protective Knee Pads, Thick Sponge Anti-Slip Knee Sleeve</t>
         </is>
       </c>
       <c r="D43" s="33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E43" s="34" t="n">
-        <v>8.99</v>
+        <v>15.99</v>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>$2-4 thrift</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="G43" s="11" t="n">
@@ -11086,7 +11086,7 @@
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>GPAA forum members discussing favorite knee pads note basic foam gardening pads work fine for short sessions, though some complain the straps can cut into legs over long days.</t>
+          <t>Captain's pick 2026-09-23, replacing the flat foam gardening pad research flagged as not moving with you on uneven creek rock -- a strap-on sleeve that stays on through repeated kneel/reposition.</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
@@ -22849,28 +22849,28 @@
       </c>
       <c r="D113" s="37" t="inlineStr">
         <is>
-          <t>Showa</t>
+          <t>Glacier Glove</t>
         </is>
       </c>
       <c r="E113" s="37" t="inlineStr">
         <is>
-          <t>Atlas 620 PVC-Coated Gauntlet Glove</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="F113" s="39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G113" s="38" t="inlineStr">
         <is>
-          <t>per pair, estimate from similar PVC gauntlet gloves</t>
+          <t>per pair, 2mm neoprene glove</t>
         </is>
       </c>
       <c r="H113" s="40" t="n">
-        <v>17.37</v>
+        <v>24.99</v>
       </c>
       <c r="I113" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/620-Coated-Liquid-Chemical-Resistant/dp/B002PJ0WRK</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="J113" s="38" t="inlineStr">
@@ -22880,17 +22880,17 @@
       </c>
       <c r="K113" s="38" t="inlineStr">
         <is>
-          <t>Amazon, Palmflex, Magid</t>
+          <t>Glacier Outdoor, Amazon</t>
         </is>
       </c>
       <c r="L113" s="38" t="inlineStr">
         <is>
-          <t>TreasureNet and prospecting forums repeatedly recommend cheap PVC-dipped work gloves like the Atlas 620 for cold-water panning — a fleece-lined double-dipped PVC glove originally designed for the Alaskan fishing trade, giving real cold/wet protection for around $10.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="M113" s="38" t="inlineStr">
         <is>
-          <t>https://www.treasurenet.com/threads/prospecting-gloves-advice.379227/, https://www.amazon.com/SHOWA-Showa-620L-09-1-Pair/dp/B000VNO2BE</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="N113" s="38" t="inlineStr">
@@ -22916,7 +22916,7 @@
       </c>
       <c r="S113" s="38" t="inlineStr">
         <is>
-          <t>Order true to hand size; too small and they crack, too large and dexterity for panning suffers. Replacement listing is the same Atlas 620 model, Small/Orange, from a different seller (original ASIN listing no longer has a valid buyable price). | TIER ODDITY: Budget ($17.37) costs more than Value ($14.99) in this category -- kept as sourced.</t>
+          <t>Order true to hand size; too small and they crack, too large and dexterity for panning suffers. Replacement listing is the same Atlas 620 model, Small/Orange, from a different seller (original ASIN listing no longer has a valid buyable price).</t>
         </is>
       </c>
       <c r="T113">
@@ -22942,28 +22942,28 @@
       </c>
       <c r="D114" s="37" t="inlineStr">
         <is>
-          <t>SE / Prospector's Choice</t>
+          <t>Glacier Glove</t>
         </is>
       </c>
       <c r="E114" s="37" t="inlineStr">
         <is>
-          <t>24" Rubber Gauntlet Gloves, Texturized Palm</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="F114" s="39" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G114" s="38" t="inlineStr">
         <is>
-          <t>per pair, per product listing</t>
+          <t>per pair, 2mm neoprene glove</t>
         </is>
       </c>
       <c r="H114" s="40" t="n">
-        <v>14.99</v>
+        <v>24.99</v>
       </c>
       <c r="I114" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/SE-GP3-RG60-Prospectors-Choice-Rubber/dp/B06XJDFYWS</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="J114" s="38" t="inlineStr">
@@ -22973,17 +22973,17 @@
       </c>
       <c r="K114" s="38" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Glacier Outdoor, Amazon</t>
         </is>
       </c>
       <c r="L114" s="38" t="inlineStr">
         <is>
-          <t>Purpose-marketed for gold panning specifically, with a longer 24" gauntlet that leaves interior room for a thin knit or fleece glove liner underneath for extra warmth in cold conditions — a step up from generic work gloves at a similar price.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="M114" s="38" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/SE-GP3-RG60-Prospectors-Choice-Rubber/dp/B06XJDFYWS</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="N114" s="38" t="inlineStr">
@@ -23009,7 +23009,7 @@
       </c>
       <c r="S114" s="38" t="inlineStr">
         <is>
-          <t>Pair with a thin liner glove for the coldest mornings | TIER ODDITY: Value ($14.99) is cheaper than Budget ($17.37) in this category -- kept as sourced.</t>
+          <t>Pair with a thin liner glove for the coldest mornings</t>
         </is>
       </c>
       <c r="T114">
@@ -23492,48 +23492,48 @@
       </c>
       <c r="D120" s="37" t="inlineStr">
         <is>
-          <t>Hodgman</t>
+          <t>FROGG TOGGS</t>
         </is>
       </c>
       <c r="E120" s="37" t="inlineStr">
         <is>
-          <t>Mackenzie Cleated Hip Bootfoot Fishing Wader</t>
+          <t>Canyon II Stockingfoot Hip Wader, Medium (needs separate wading shoe)</t>
         </is>
       </c>
       <c r="F120" s="39" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="G120" s="38" t="inlineStr">
         <is>
-          <t>~3 lb, typical neoprene hip wader pair</t>
+          <t>category estimate, no vendor spec published -- 4-ply nylon, no attached boot</t>
         </is>
       </c>
       <c r="H120" s="40" t="n">
-        <v>43.51</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="I120" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/Hodgman-Mackenzie-Cleated-Hip-Bootfoot-Fishing-Wader/43927288</t>
+          <t>https://www.amazon.com/Frogg-Toggs-Canyon-Breathable-Stockingfoot/dp/B07FKMB1DB</t>
         </is>
       </c>
       <c r="J120" s="38" t="inlineStr">
         <is>
-          <t>$20-30 used</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="K120" s="38" t="inlineStr">
         <is>
-          <t>Walmart, Bass Pro</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="L120" s="38" t="inlineStr">
         <is>
-          <t>Hip waders show up in wading/fishing gear guides as an affordable step up for anyone who wants to stand in deeper pools without soaking pants — useful if scouting deeper holes, though most panning happens in water too shallow to need them.</t>
+          <t>Breathable upgrade over the rubber/PVC Hodgman pick -- highest-rated breathable hip wader at this size, and hip height already exceeds what shin-deep hand-panning needs. Needs a separate wading shoe (not bundled).</t>
         </is>
       </c>
       <c r="M120" s="38" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/Hodgman-Mackenzie-Cleated-Hip-Bootfoot-Fishing-Wader/43927288</t>
+          <t>https://www.froggtoggs.com/canyon-ii-stockingfoot-breathable-hip-wader</t>
         </is>
       </c>
       <c r="N120" s="38" t="inlineStr">
@@ -23678,48 +23678,48 @@
       </c>
       <c r="D122" s="37" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Bodyprox</t>
         </is>
       </c>
       <c r="E122" s="37" t="inlineStr">
         <is>
-          <t>Foam Gardening Knee Pad</t>
+          <t>Protective Knee Pads, Thick Sponge Anti-Slip Knee Sleeve</t>
         </is>
       </c>
       <c r="F122" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G122" s="38" t="inlineStr">
         <is>
-          <t>per pair, standard foam kneeler</t>
+          <t>per pair, strap-on sleeve</t>
         </is>
       </c>
       <c r="H122" s="40" t="n">
-        <v>8.99</v>
+        <v>15.99</v>
       </c>
       <c r="I122" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Fiskars-94216974J-Ultralight-Kneeling-Cushion/dp/B0002YTVJA</t>
+          <t>https://www.amazon.com/gp/product/B01L379FPE</t>
         </is>
       </c>
       <c r="J122" s="38" t="inlineStr">
         <is>
-          <t>$2-4 thrift</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="K122" s="38" t="inlineStr">
         <is>
-          <t>Walmart, hardware store</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="L122" s="38" t="inlineStr">
         <is>
-          <t>GPAA forum members discussing favorite knee pads note basic foam gardening pads work fine for short sessions, though some complain the straps can cut into legs over long days.</t>
+          <t>Captain's pick 2026-09-23, replacing the flat foam gardening pad research flagged as not moving with you on uneven creek rock -- a strap-on sleeve that stays on through repeated kneel/reposition.</t>
         </is>
       </c>
       <c r="M122" s="38" t="inlineStr">
         <is>
-          <t>https://www.goldprospectors.org/Forum/aft/9275</t>
+          <t>https://www.amazon.com/gp/product/B01L379FPE</t>
         </is>
       </c>
       <c r="N122" s="38" t="inlineStr">

</xml_diff>

<commit_message>
Set Jordan's picks for gloves/knee-pads/waders, rebuild buy list
Glacier Glove Kenai Original neoprene gloves ($24.99, dexterity over
staying dry), Bodyprox strap-on knee pads ($15.99, Jordan's own find),
Frogg Toggs Canyon II breathable hip waders ($98.29, upgrade from the
rubber/PVC Hodgman pick). Live prices verified in-browser. Rebuilt via
build_gear_picker.py -> build_buy_list.py -> build_hub.py.
</commit_message>
<xml_diff>
--- a/Gear_Picker.xlsx
+++ b/Gear_Picker.xlsx
@@ -10675,14 +10675,14 @@
       </c>
       <c r="C40" s="32" t="inlineStr">
         <is>
-          <t>Atlas 620 PVC-Coated Gauntlet Glove</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E40" s="34" t="n">
-        <v>17.37</v>
+        <v>24.99</v>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>TreasureNet and prospecting forums repeatedly recommend cheap PVC-dipped work gloves like the Atlas 620 for cold-water panning — a fleece-lined double-dipped PVC glove originally designed for the Alaskan fishing trade, giving real cold/wet protection for around $10.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
@@ -10714,14 +10714,14 @@
       </c>
       <c r="L40" s="35" t="inlineStr">
         <is>
-          <t>24" Rubber Gauntlet Gloves, Texturized Palm</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="M40" s="33" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N40" s="34" t="n">
-        <v>14.99</v>
+        <v>24.99</v>
       </c>
       <c r="O40" s="11" t="inlineStr">
         <is>
@@ -10738,7 +10738,7 @@
       </c>
       <c r="R40" s="11" t="inlineStr">
         <is>
-          <t>Purpose-marketed for gold panning specifically, with a longer 24" gauntlet that leaves interior room for a thin knit or fleece glove liner underneath for extra warmth in cold conditions — a step up from generic work gloves at a similar price.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="S40" s="11" t="inlineStr">
@@ -10972,18 +10972,18 @@
       </c>
       <c r="L42" s="35" t="inlineStr">
         <is>
-          <t>Mackenzie Cleated Hip Bootfoot Fishing Wader</t>
+          <t>Canyon II Stockingfoot Hip Wader, Medium (needs separate wading shoe)</t>
         </is>
       </c>
       <c r="M42" s="33" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="N42" s="34" t="n">
-        <v>43.51</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="O42" s="11" t="inlineStr">
         <is>
-          <t>$20-30 used</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="P42" s="11" t="n">
@@ -10996,7 +10996,7 @@
       </c>
       <c r="R42" s="11" t="inlineStr">
         <is>
-          <t>Hip waders show up in wading/fishing gear guides as an affordable step up for anyone who wants to stand in deeper pools without soaking pants — useful if scouting deeper holes, though most panning happens in water too shallow to need them.</t>
+          <t>Breathable upgrade over the rubber/PVC Hodgman pick -- highest-rated breathable hip wader at this size, and hip height already exceeds what shin-deep hand-panning needs. Needs a separate wading shoe (not bundled).</t>
         </is>
       </c>
       <c r="S42" s="11" t="inlineStr">
@@ -11062,18 +11062,18 @@
       </c>
       <c r="C43" s="32" t="inlineStr">
         <is>
-          <t>Foam Gardening Knee Pad</t>
+          <t>Protective Knee Pads, Thick Sponge Anti-Slip Knee Sleeve</t>
         </is>
       </c>
       <c r="D43" s="33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E43" s="34" t="n">
-        <v>8.99</v>
+        <v>15.99</v>
       </c>
       <c r="F43" s="11" t="inlineStr">
         <is>
-          <t>$2-4 thrift</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="G43" s="11" t="n">
@@ -11086,7 +11086,7 @@
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>GPAA forum members discussing favorite knee pads note basic foam gardening pads work fine for short sessions, though some complain the straps can cut into legs over long days.</t>
+          <t>Captain's pick 2026-09-23, replacing the flat foam gardening pad research flagged as not moving with you on uneven creek rock -- a strap-on sleeve that stays on through repeated kneel/reposition.</t>
         </is>
       </c>
       <c r="J43" s="11" t="inlineStr">
@@ -22849,28 +22849,28 @@
       </c>
       <c r="D113" s="37" t="inlineStr">
         <is>
-          <t>Showa</t>
+          <t>Glacier Glove</t>
         </is>
       </c>
       <c r="E113" s="37" t="inlineStr">
         <is>
-          <t>Atlas 620 PVC-Coated Gauntlet Glove</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="F113" s="39" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G113" s="38" t="inlineStr">
         <is>
-          <t>per pair, estimate from similar PVC gauntlet gloves</t>
+          <t>per pair, 2mm neoprene glove</t>
         </is>
       </c>
       <c r="H113" s="40" t="n">
-        <v>17.37</v>
+        <v>24.99</v>
       </c>
       <c r="I113" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/620-Coated-Liquid-Chemical-Resistant/dp/B002PJ0WRK</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="J113" s="38" t="inlineStr">
@@ -22880,17 +22880,17 @@
       </c>
       <c r="K113" s="38" t="inlineStr">
         <is>
-          <t>Amazon, Palmflex, Magid</t>
+          <t>Glacier Outdoor, Amazon</t>
         </is>
       </c>
       <c r="L113" s="38" t="inlineStr">
         <is>
-          <t>TreasureNet and prospecting forums repeatedly recommend cheap PVC-dipped work gloves like the Atlas 620 for cold-water panning — a fleece-lined double-dipped PVC glove originally designed for the Alaskan fishing trade, giving real cold/wet protection for around $10.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="M113" s="38" t="inlineStr">
         <is>
-          <t>https://www.treasurenet.com/threads/prospecting-gloves-advice.379227/, https://www.amazon.com/SHOWA-Showa-620L-09-1-Pair/dp/B000VNO2BE</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="N113" s="38" t="inlineStr">
@@ -22916,7 +22916,7 @@
       </c>
       <c r="S113" s="38" t="inlineStr">
         <is>
-          <t>Order true to hand size; too small and they crack, too large and dexterity for panning suffers. Replacement listing is the same Atlas 620 model, Small/Orange, from a different seller (original ASIN listing no longer has a valid buyable price). | TIER ODDITY: Budget ($17.37) costs more than Value ($14.99) in this category -- kept as sourced.</t>
+          <t>Order true to hand size; too small and they crack, too large and dexterity for panning suffers. Replacement listing is the same Atlas 620 model, Small/Orange, from a different seller (original ASIN listing no longer has a valid buyable price).</t>
         </is>
       </c>
       <c r="T113">
@@ -22942,28 +22942,28 @@
       </c>
       <c r="D114" s="37" t="inlineStr">
         <is>
-          <t>SE / Prospector's Choice</t>
+          <t>Glacier Glove</t>
         </is>
       </c>
       <c r="E114" s="37" t="inlineStr">
         <is>
-          <t>24" Rubber Gauntlet Gloves, Texturized Palm</t>
+          <t>Kenai Original</t>
         </is>
       </c>
       <c r="F114" s="39" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G114" s="38" t="inlineStr">
         <is>
-          <t>per pair, per product listing</t>
+          <t>per pair, 2mm neoprene glove</t>
         </is>
       </c>
       <c r="H114" s="40" t="n">
-        <v>14.99</v>
+        <v>24.99</v>
       </c>
       <c r="I114" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/SE-GP3-RG60-Prospectors-Choice-Rubber/dp/B06XJDFYWS</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="J114" s="38" t="inlineStr">
@@ -22973,17 +22973,17 @@
       </c>
       <c r="K114" s="38" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Glacier Outdoor, Amazon</t>
         </is>
       </c>
       <c r="L114" s="38" t="inlineStr">
         <is>
-          <t>Purpose-marketed for gold panning specifically, with a longer 24" gauntlet that leaves interior room for a thin knit or fleece glove liner underneath for extra warmth in cold conditions — a step up from generic work gloves at a similar price.</t>
+          <t>Captain's pick 2026-09-23: 35-year standard for cold fly-fishing, 2mm fleece-lined neoprene with a sharkskin palm -- chose dexterity (feel the pan, pick gravel) over staying bone-dry.</t>
         </is>
       </c>
       <c r="M114" s="38" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/SE-GP3-RG60-Prospectors-Choice-Rubber/dp/B06XJDFYWS</t>
+          <t>https://glacieroutdoor.com/products/kenai-original</t>
         </is>
       </c>
       <c r="N114" s="38" t="inlineStr">
@@ -23009,7 +23009,7 @@
       </c>
       <c r="S114" s="38" t="inlineStr">
         <is>
-          <t>Pair with a thin liner glove for the coldest mornings | TIER ODDITY: Value ($14.99) is cheaper than Budget ($17.37) in this category -- kept as sourced.</t>
+          <t>Pair with a thin liner glove for the coldest mornings</t>
         </is>
       </c>
       <c r="T114">
@@ -23492,48 +23492,48 @@
       </c>
       <c r="D120" s="37" t="inlineStr">
         <is>
-          <t>Hodgman</t>
+          <t>FROGG TOGGS</t>
         </is>
       </c>
       <c r="E120" s="37" t="inlineStr">
         <is>
-          <t>Mackenzie Cleated Hip Bootfoot Fishing Wader</t>
+          <t>Canyon II Stockingfoot Hip Wader, Medium (needs separate wading shoe)</t>
         </is>
       </c>
       <c r="F120" s="39" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="G120" s="38" t="inlineStr">
         <is>
-          <t>~3 lb, typical neoprene hip wader pair</t>
+          <t>category estimate, no vendor spec published -- 4-ply nylon, no attached boot</t>
         </is>
       </c>
       <c r="H120" s="40" t="n">
-        <v>43.51</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="I120" s="41" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/Hodgman-Mackenzie-Cleated-Hip-Bootfoot-Fishing-Wader/43927288</t>
+          <t>https://www.amazon.com/Frogg-Toggs-Canyon-Breathable-Stockingfoot/dp/B07FKMB1DB</t>
         </is>
       </c>
       <c r="J120" s="38" t="inlineStr">
         <is>
-          <t>$20-30 used</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="K120" s="38" t="inlineStr">
         <is>
-          <t>Walmart, Bass Pro</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="L120" s="38" t="inlineStr">
         <is>
-          <t>Hip waders show up in wading/fishing gear guides as an affordable step up for anyone who wants to stand in deeper pools without soaking pants — useful if scouting deeper holes, though most panning happens in water too shallow to need them.</t>
+          <t>Breathable upgrade over the rubber/PVC Hodgman pick -- highest-rated breathable hip wader at this size, and hip height already exceeds what shin-deep hand-panning needs. Needs a separate wading shoe (not bundled).</t>
         </is>
       </c>
       <c r="M120" s="38" t="inlineStr">
         <is>
-          <t>https://www.walmart.com/ip/Hodgman-Mackenzie-Cleated-Hip-Bootfoot-Fishing-Wader/43927288</t>
+          <t>https://www.froggtoggs.com/canyon-ii-stockingfoot-breathable-hip-wader</t>
         </is>
       </c>
       <c r="N120" s="38" t="inlineStr">
@@ -23678,48 +23678,48 @@
       </c>
       <c r="D122" s="37" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Bodyprox</t>
         </is>
       </c>
       <c r="E122" s="37" t="inlineStr">
         <is>
-          <t>Foam Gardening Knee Pad</t>
+          <t>Protective Knee Pads, Thick Sponge Anti-Slip Knee Sleeve</t>
         </is>
       </c>
       <c r="F122" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G122" s="38" t="inlineStr">
         <is>
-          <t>per pair, standard foam kneeler</t>
+          <t>per pair, strap-on sleeve</t>
         </is>
       </c>
       <c r="H122" s="40" t="n">
-        <v>8.99</v>
+        <v>15.99</v>
       </c>
       <c r="I122" s="41" t="inlineStr">
         <is>
-          <t>https://www.amazon.com/Fiskars-94216974J-Ultralight-Kneeling-Cushion/dp/B0002YTVJA</t>
+          <t>https://www.amazon.com/gp/product/B01L379FPE</t>
         </is>
       </c>
       <c r="J122" s="38" t="inlineStr">
         <is>
-          <t>$2-4 thrift</t>
+          <t>n/a, cheap enough to buy new</t>
         </is>
       </c>
       <c r="K122" s="38" t="inlineStr">
         <is>
-          <t>Walmart, hardware store</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="L122" s="38" t="inlineStr">
         <is>
-          <t>GPAA forum members discussing favorite knee pads note basic foam gardening pads work fine for short sessions, though some complain the straps can cut into legs over long days.</t>
+          <t>Captain's pick 2026-09-23, replacing the flat foam gardening pad research flagged as not moving with you on uneven creek rock -- a strap-on sleeve that stays on through repeated kneel/reposition.</t>
         </is>
       </c>
       <c r="M122" s="38" t="inlineStr">
         <is>
-          <t>https://www.goldprospectors.org/Forum/aft/9275</t>
+          <t>https://www.amazon.com/gp/product/B01L379FPE</t>
         </is>
       </c>
       <c r="N122" s="38" t="inlineStr">

</xml_diff>